<commit_message>
Visor: lodosa (2026-10-21 21:07)
</commit_message>
<xml_diff>
--- a/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
+++ b/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
@@ -1258,7 +1258,7 @@
     <t xml:space="preserve">Tablero OSB/3 hidrófugo de 20 mm fijado mecánicamente a la losa a través del aislamiento.</t>
   </si>
   <si>
-    <t xml:space="preserve">Medición del IFC final (opción 3, 21-oct): igual que la teja, faldones 81,23 + aleros 6,31 m²</t>
+    <t xml:space="preserve">Medición del IFC final (opción 3, 21-oct): igual que la teja, faldones 82,06 + aleros 6,31 m²</t>
   </si>
   <si>
     <t xml:space="preserve">07.03</t>
@@ -3784,7 +3784,7 @@
     <t xml:space="preserve">Opción 3 de cubiertas · IFC final (21-oct)</t>
   </si>
   <si>
-    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261021-1843.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 30,02 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (81,23 m²); OSB, lámina, rastreles y teja, con ellos (87,54 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (308,49 m², huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta hasta la pared (24,39 m en total). La unidad exterior de la aerotermia vuelve a la cubierta plana. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement).</t>
+    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261021-2001.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (322,29 m², con 13,43 m² de cantos de losas y faldones que quedaban vistos; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta hasta la pared (24,39 m en total). La unidad exterior de la aerotermia vuelve a la cubierta plana. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement).</t>
   </si>
   <si>
     <t xml:space="preserve">MEDICIONES DEL MODELO BIM FRENTE A LA PROPUESTA DE OCTUBRE</t>
@@ -3826,16 +3826,16 @@
     <t xml:space="preserve">Superficie de estancias y escalera de planta baja (garaje incluido)</t>
   </si>
   <si>
-    <t xml:space="preserve">Forjado de viguetas 20+5 en todo (Enrique 14-oct), del BIM en proyección con los zunchos de forjado dentro y sin huecos de escalera ni patio: primera 123.4 (con el techo del garaje 53.8) + segunda con la terraza 102.4 + cubierta plana 49.3. El pilar de hormigón junto a la escalera (27×81, tres plantas, 1.87 m³) no tiene partida · Menos la terraza de planta segunda, 11.1 m², que pasa a 15+5 (05.02.11) · Opción 2 de cubiertas (16-oct): la cubierta plana del BIM pasa de 49,3 a 46,47 m² (+11,33 de la tira que deja de ser faldón, −14,17 del faldón nuevo sobre la escalera); los 17,15 m² bajo el faldón nuevo de C. del Peso conservan el forjado · Opción 3 de cubiertas, IFC final (21-oct): la cubierta plana pasa de 46,47 a 30,02 m²; los 16,45 m² restantes son ahora el faldón a la medianera oeste (losa de Ytong), sin forjado: 261,19 − 16,45</t>
+    <t xml:space="preserve">Forjado de viguetas 20+5 en todo (Enrique 14-oct), del BIM en proyección con los zunchos de forjado dentro y sin huecos de escalera ni patio: primera 123.4 (con el techo del garaje 53.8) + segunda con la terraza 102.4 + cubierta plana 49.3. El pilar de hormigón junto a la escalera (27×81, tres plantas, 1.87 m³) no tiene partida · Menos la terraza de planta segunda, 11.1 m², que pasa a 15+5 (05.02.11) · Opción 2 de cubiertas (16-oct): la cubierta plana del BIM pasa de 49,3 a 46,47 m² (+11,33 de la tira que deja de ser faldón, −14,17 del faldón nuevo sobre la escalera); los 17,15 m² bajo el faldón nuevo de C. del Peso conservan el forjado · Opción 3 de cubiertas, IFC final (21-oct): la cubierta plana pasa de 46,47 a 30,02 m²; los 16,45 m² restantes son ahora el faldón a la medianera oeste (losa de Ytong), sin forjado: 261,19 − 16,45 · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): cubierta plana 29,31 m² (planta de cubiertas de Enrique, 21-oct 18:50): 261,19 − 17,16</t>
   </si>
   <si>
     <t xml:space="preserve">Sin losa maciza: el techo del garaje también es forjado de viguetas y está medido en 05.02.01 (Enrique 14-oct)</t>
   </si>
   <si>
-    <t xml:space="preserve">Zunchos de forjado sobre muros de carga (147.9 m, 14.6 m³) y de coronación bajo cubierta (69.4 m, 3.6 m³, canto supuesto 25 cm) · Opción 2 de cubiertas (16-oct): zunchos remedidos en el BIM de la opción 2 · Opción 3 de cubiertas, IFC final (21-oct): zunchos remedidos en el modelo de la opción 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faldones medidos en pendiente (sin aleros, 6.0 m² en planta aparte) · Opción 2 de cubiertas (16-oct): faldones en pendiente 62,44 + faldón sobre la escalera 14,79 + faldón de C. del Peso sobre la cubierta plana 17,90 − tira que pasa a plana 11,84 · Opción 3 de cubiertas, IFC final (21-oct): faldón de C. Ancha 47,37 (con el de la escalera, mismo plano) + faldón de C. del Peso 11,58 + faldón a la medianera oeste 22,28 = 81,23 m² en pendiente, sin los aleros: regla de Enrique del 21-oct, el alero es parte de su faldón pero vuela 200 mm sin aislamiento (no lleva losa de Ytong ni XPS). Ya no hay faldón ventilado</t>
+    <t xml:space="preserve">Zunchos de forjado sobre muros de carga (147.9 m, 14.6 m³) y de coronación bajo cubierta (69.4 m, 3.6 m³, canto supuesto 25 cm) · Opción 2 de cubiertas (16-oct): zunchos remedidos en el BIM de la opción 2 · Opción 3 de cubiertas, IFC final (21-oct): zunchos remedidos en el modelo de la opción 3 · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): zunchos remedidos en el modelo de la opción 3 (IFC 20:01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faldones medidos en pendiente (sin aleros, 6.0 m² en planta aparte) · Opción 2 de cubiertas (16-oct): faldones en pendiente 62,44 + faldón sobre la escalera 14,79 + faldón de C. del Peso sobre la cubierta plana 17,90 − tira que pasa a plana 11,84 · Opción 3 de cubiertas, IFC final (21-oct): faldón de C. Ancha 47,37 (con el de la escalera, mismo plano) + faldón de C. del Peso 11,58 + faldón a la medianera oeste 22,28 = 81,23 m² en pendiente, sin los aleros: regla de Enrique del 21-oct, el alero es parte de su faldón pero vuela 200 mm sin aislamiento (no lleva losa de Ytong ni XPS). Ya no hay faldón ventilado · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): faldón de C. Ancha 47,38 + faldón de C. del Peso 11,54 + faldón a la medianera oeste 23,14 = 82,06 m² en pendiente, sin los aleros (200 mm sin aislamiento): planta de cubiertas de Enrique del 21-oct (la limatesa va a la esquina del alero en la medianera, faldón oeste al 21 %; su borde norte llega 22 cm más allá)</t>
   </si>
   <si>
     <t xml:space="preserve">Pilar de 27×81 en baja, primera y segunda, del suelo a la cara inferior del forjado de encima · Partida nueva</t>
@@ -3844,40 +3844,40 @@
     <t xml:space="preserve">Forjado de la terraza de planta segunda en el BIM (15+5, Enrique 14-oct) · Partida nueva</t>
   </si>
   <si>
-    <t xml:space="preserve">Muros M1/M9 de fachada: longitud de eje × altura real de cada tramo, sin huecos ni zócalo · Opción 3 de cubiertas, IFC final (21-oct): −0,71 m²: los muros se acortan o adelgazan 15 mm para dejar paso al revoco continuo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros M6/M7/M8/M14 a patio o sin casa pegada · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro (M7e) que cambia con los faldones nuevos · +13,89 m² de piñones de Ytong 20 cm que cierran el faldón de C. del Peso sobre la cubierta plana (cara norte 2,97 × 2,16 m y cara este 5,81 m de 0,42 a 2,16 m) · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte (2,97 × 2,16 m); queda el piñón este (7,47 m²) · Opción 3 de cubiertas, IFC final (21-oct): sin el faldón ventilado de C. del Peso: −20,86 m² de muros con las dos caras al exterior (M7e) y −11,22 m² de M6/M7 de segunda; +13,73 m² de muros de quiebro (M7c) donde la cubierta alta se junta con la baja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medianeras M2–M5/M10–M12 e interiores de carga M13 · Opción 2 de cubiertas (16-oct): +8,09 m² de medianera M2 que sube hasta el faldón sobre la escalera y +2,54 m² de M13 (muro de la escalera hasta el alféizar del ventanal y dintel encima) · Opción 3 de cubiertas, IFC final (21-oct): +7,09 m² de la medianera M2 que sube hasta el faldón a la medianera oeste, +2,62 m² de muro de carga M13/M13b y −0,37 m² de recortes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capa de junta de los muros de medianera · Opción 2 de cubiertas (16-oct): +8,09 m² de la medianera M2 que sube hasta el faldón sobre la escalera · Opción 3 de cubiertas, IFC final (21-oct): +6,72 m² de junta de las medianeras (la M2 que sube). Se mide con la geometría. En el IFC 1843 la junta sale en todas las medianeras como capa del muro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros M4/M5/M6 (trasdosado de 7 cm con cámara) · Opción 3 de cubiertas, IFC final (21-oct): −2,09 m² (M6 de primera y segunda)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabiques T1/T2/T3 · Opción 2 de cubiertas (16-oct): −2,36 m²: el tabique T2 bajo la tira, que pasa a cubierta plana, es más bajo · Opción 3 de cubiertas, IFC final (21-oct): −0,20 m² de recortes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frentes de forjado revestidos en los bordes exteriores de los forjados · Opción 2 de cubiertas (16-oct): +1,87 m de frente de forjado junto a la escalera · Opción 3 de cubiertas, IFC final (21-oct): frentes de forjado remedidos: −5,76 m (la cubierta plana que pasa a faldón y el recorte de 15 mm del revoco)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faldones en pendiente · Opción 2 de cubiertas (16-oct): igual que 05.02.07 · Faldón de C. del Peso ventilado (Enrique 16-oct): sin XPS en sus 17,90 m²; el aislamiento va en la cubierta plana de debajo · Opción 3 de cubiertas, IFC final (21-oct): igual que 05.02.07, sin los aleros: todos los faldones llevan XPS 10 cm (ya no hay faldón ventilado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faldones en pendiente (los aleros se miden aparte) · Opción 2 de cubiertas (16-oct): igual que 05.02.07 · Opción 3 de cubiertas, IFC final (21-oct): faldones 81,23 m² en pendiente + aleros 6,31 m² (3,17 C. Ancha + 3,02 C. del Peso + 0,12 medianera oeste): la teja, la lámina, el OSB y los rastreles llegan al borde del alero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XPS 14 cm de la cubierta plana del BIM (49.3 m²). Sustituye a la cubierta invertida: no hay ninguna (Enrique 14-oct); el resto del paquete está en 05.02.01 (forjado), 08.02 (XPS 4 en patio, porche y terraza), 08.03 (antiimpacto), 07.12 (pendientes), 08.08 (lámina), 10.09 (mortero de protección) y 10.04 (microcemento) · La propuesta medía 77,3 m² de cubierta invertida a 74 €/m² (5.720,20 €) · Opción 2 de cubiertas (16-oct): solo la cubierta plana descubierta: 46,47 − 17,15 m² bajo el faldón de C. del Peso, que lleva el aislamiento en el faldón · Faldón de C. del Peso ventilado (Enrique 16-oct): la cubierta plana bajo él (17,15 m²) lleva el XPS de 14 cm: 29,32 + 17,15 · Opción 3 de cubiertas, IFC final (21-oct): cubierta plana del IFC, 30,02 m² (ya no hay cubierta plana bajo un faldón)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón, que es suelo del almacenaje y de la aerotermia · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubierta plana 49.3 + patio y porche 29.6 m² (bajo el XPS) · Partida nueva · Opción 2 de cubiertas (16-oct): cubierta plana descubierta 29,32 + patio y porche 29,6 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): cubierta plana 30,02 + patio y porche 29,65 m²</t>
+    <t xml:space="preserve">Muros M1/M9 de fachada: longitud de eje × altura real de cada tramo, sin huecos ni zócalo · Opción 3 de cubiertas, IFC final (21-oct): −0,71 m²: los muros se acortan o adelgazan 15 mm para dejar paso al revoco continuo · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +0,52 m² de fachada con las dos caras al exterior (M1e) en segunda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros M6/M7/M8/M14 a patio o sin casa pegada · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro (M7e) que cambia con los faldones nuevos · +13,89 m² de piñones de Ytong 20 cm que cierran el faldón de C. del Peso sobre la cubierta plana (cara norte 2,97 × 2,16 m y cara este 5,81 m de 0,42 a 2,16 m) · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte (2,97 × 2,16 m); queda el piñón este (7,47 m²) · Opción 3 de cubiertas, IFC final (21-oct): sin el faldón ventilado de C. del Peso: −20,86 m² de muros con las dos caras al exterior (M7e) y −11,22 m² de M6/M7 de segunda; +13,73 m² de muros de quiebro (M7c) donde la cubierta alta se junta con la baja · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +0,89 m² de muros exteriores de segunda (M6, M7, M7c, M8) con la planta de cubiertas nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medianeras M2–M5/M10–M12 e interiores de carga M13 · Opción 2 de cubiertas (16-oct): +8,09 m² de medianera M2 que sube hasta el faldón sobre la escalera y +2,54 m² de M13 (muro de la escalera hasta el alféizar del ventanal y dintel encima) · Opción 3 de cubiertas, IFC final (21-oct): +7,09 m² de la medianera M2 que sube hasta el faldón a la medianera oeste, +2,62 m² de muro de carga M13/M13b y −0,37 m² de recortes · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): −1,49 m²: el muro de 45 cm del baño de segunda y de la cocina pasa a ser de carga de 20 cm + trasdosado (M13t, Enrique 21-oct), medianeras y muros de carga remedidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capa de junta de los muros de medianera · Opción 2 de cubiertas (16-oct): +8,09 m² de la medianera M2 que sube hasta el faldón sobre la escalera · Opción 3 de cubiertas, IFC final (21-oct): +6,72 m² de junta de las medianeras (la M2 que sube). Se mide con la geometría. En el IFC 1843 la junta sale en todas las medianeras como capa del muro · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): −0,23 m² de medianera de segunda (IFC 20:01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros M4/M5/M6 (trasdosado de 7 cm con cámara) · Opción 3 de cubiertas, IFC final (21-oct): −2,09 m² (M6 de primera y segunda) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +3,60 m² del trasdosado del muro de carga del baño de segunda y de la cocina (M13t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabiques T1/T2/T3 · Opción 2 de cubiertas (16-oct): −2,36 m²: el tabique T2 bajo la tira, que pasa a cubierta plana, es más bajo · Opción 3 de cubiertas, IFC final (21-oct): −0,20 m² de recortes · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +1,80 m² de tabiques de segunda con la planta de cubiertas nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frentes de forjado revestidos en los bordes exteriores de los forjados · Opción 2 de cubiertas (16-oct): +1,87 m de frente de forjado junto a la escalera · Opción 3 de cubiertas, IFC final (21-oct): frentes de forjado remedidos: −5,76 m (la cubierta plana que pasa a faldón y el recorte de 15 mm del revoco) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): frentes de forjado remedidos: −0,80 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faldones en pendiente · Opción 2 de cubiertas (16-oct): igual que 05.02.07 · Faldón de C. del Peso ventilado (Enrique 16-oct): sin XPS en sus 17,90 m²; el aislamiento va en la cubierta plana de debajo · Opción 3 de cubiertas, IFC final (21-oct): igual que 05.02.07, sin los aleros: todos los faldones llevan XPS 10 cm (ya no hay faldón ventilado) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): igual que 05.02.07, sin los aleros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faldones en pendiente (los aleros se miden aparte) · Opción 2 de cubiertas (16-oct): igual que 05.02.07 · Opción 3 de cubiertas, IFC final (21-oct): faldones 81,23 m² en pendiente + aleros 6,31 m² (3,17 C. Ancha + 3,02 C. del Peso + 0,12 medianera oeste): la teja, la lámina, el OSB y los rastreles llegan al borde del alero · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): faldones 82,06 m² en pendiente + aleros 6,31 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XPS 14 cm de la cubierta plana del BIM (49.3 m²). Sustituye a la cubierta invertida: no hay ninguna (Enrique 14-oct); el resto del paquete está en 05.02.01 (forjado), 08.02 (XPS 4 en patio, porche y terraza), 08.03 (antiimpacto), 07.12 (pendientes), 08.08 (lámina), 10.09 (mortero de protección) y 10.04 (microcemento) · La propuesta medía 77,3 m² de cubierta invertida a 74 €/m² (5.720,20 €) · Opción 2 de cubiertas (16-oct): solo la cubierta plana descubierta: 46,47 − 17,15 m² bajo el faldón de C. del Peso, que lleva el aislamiento en el faldón · Faldón de C. del Peso ventilado (Enrique 16-oct): la cubierta plana bajo él (17,15 m²) lleva el XPS de 14 cm: 29,32 + 17,15 · Opción 3 de cubiertas, IFC final (21-oct): cubierta plana del IFC, 30,02 m² (ya no hay cubierta plana bajo un faldón) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): cubierta plana de la planta de cubiertas de Enrique (21-oct): 29,31 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón, que es suelo del almacenaje y de la aerotermia · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 29,31 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubierta plana 49.3 + patio y porche 29.6 m² (bajo el XPS) · Partida nueva · Opción 2 de cubiertas (16-oct): cubierta plana descubierta 29,32 + patio y porche 29,6 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): cubierta plana 30,02 + patio y porche 29,65 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): cubierta plana 29,31 + patio y porche 29,65 m²</t>
   </si>
   <si>
     <t xml:space="preserve">Suelo de planta baja dentro de la envolvente (sin garaje)</t>
@@ -3886,13 +3886,13 @@
     <t xml:space="preserve">XPS 4 cm en todos los forjados: interiores, patio y porche y terraza (la cubierta plana lleva 14 cm, ver 07.09)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lámina antiimpacto en todos los forjados: interiores de primera y segunda y también patio y porche, terraza y cubierta plana (Enrique 14-oct) · Opción 2 de cubiertas (16-oct): la cubierta plana bajo el faldón de C. del Peso (17,15 m²) ya no es suelo: 240,4 − 49,3 + 29,32 · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): 240,4 − 49,3 + 30,02 (la cubierta plana del IFC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En planta: patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² (los remontes van en el precio) · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zonas con trama de la capa «falsos techos», cerradas hasta los muros · Opción 2 de cubiertas (16-oct): +8,52 m² de falso techo plano a +10,50 bajo el faldón de la escalera (cabeza del ventanal) · Opción 3 de cubiertas, IFC final (21-oct): falsos techos del IFC: 88,43 m². Bajo el faldón de la escalera ya no hay falso techo plano (−8,52 m²): el V12 llega hasta el faldón</t>
+    <t xml:space="preserve">Lámina antiimpacto en todos los forjados: interiores de primera y segunda y también patio y porche, terraza y cubierta plana (Enrique 14-oct) · Opción 2 de cubiertas (16-oct): la cubierta plana bajo el faldón de C. del Peso (17,15 m²) ya no es suelo: 240,4 − 49,3 + 29,32 · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): 240,4 − 49,3 + 30,02 (la cubierta plana del IFC) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): 240,4 − 49,3 + 29,31 (la cubierta plana)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En planta: patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² (los remontes van en el precio) · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 29,31 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zonas con trama de la capa «falsos techos», cerradas hasta los muros · Opción 2 de cubiertas (16-oct): +8,52 m² de falso techo plano a +10,50 bajo el faldón de la escalera (cabeza del ventanal) · Opción 3 de cubiertas, IFC final (21-oct): falsos techos del IFC: 88,43 m². Bajo el faldón de la escalera ya no hay falso techo plano (−8,52 m²): el V12 llega hasta el faldón · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): falsos techos del IFC 20:01</t>
   </si>
   <si>
     <t xml:space="preserve">Longitud de los bordes libres del falso techo en el BIM × altura hasta la cara inferior del forjado (0,86 m en baja, 0,42 m en primera y 0,41 m en segunda) · Partida nueva · Opción 3 de cubiertas, IFC final (21-oct): tabicas del IFC: 22,30 m², sin cambios</t>
@@ -3904,19 +3904,19 @@
     <t xml:space="preserve">Suelos interiores sin baños ni aseos</t>
   </si>
   <si>
-    <t xml:space="preserve">Patio y porche, terraza de segunda y terraza en cubierta · Opción 2 de cubiertas (16-oct): patio y porche, terraza de segunda y cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón (suelo del almacenaje y de la aerotermia) · Opción 3 de cubiertas, IFC final (21-oct): patio y porche, terraza de segunda y cubierta plana 30,02 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caras revocadas de muros exteriores y frentes de forjado · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro y +0,68 m² de frente de forjado · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): revoco continuo del IFC (piel vista de la casa, 34 paños de arriba abajo, regla de Enrique del 19 y 21-oct): caras 289,80 m² con los huecos descontados + mochetas y dinteles 18,68 m²; sin medianeras, bajo aleros ni zócalo. Sustituye a la medición por caras de muro (261,81)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paredes 726.4 m² (incluye 27.6 m² de baños y aseos por encima de 2,28 m) y techos sin falso techo 214.4 m² · Opción 2 de cubiertas (16-oct): paredes: +8,09 medianera M2, +5,08 muro M13 (dos caras), −4,72 tabique T2 (dos caras), −1,50 quiebro; techos: −8,52 m² que pasan a falso techo · Opción 3 de cubiertas, IFC final (21-oct): paredes −0,80 m² (cambios de muros de segunda) y techos +8,89 m²: bajo el faldón de la escalera ya no hay falso techo (+8,52) y el faldón a la medianera oeste tiene más superficie en pendiente que la cubierta plana a la que sustituye (+0,37)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caras de baños y aseos con baldosa hasta 2,28 m (por encima, yeso y pintura) · Opción 3 de cubiertas, IFC final (21-oct): +1,06 m² del muro M13b del baño de segunda (hasta 2,28 m). Se mide con la geometría. En el IFC 1843 la baldosa sale en los tabiques de baño (T2, M13b)</t>
+    <t xml:space="preserve">Patio y porche, terraza de segunda y terraza en cubierta · Opción 2 de cubiertas (16-oct): patio y porche, terraza de segunda y cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón (suelo del almacenaje y de la aerotermia) · Opción 3 de cubiertas, IFC final (21-oct): patio y porche, terraza de segunda y cubierta plana 30,02 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): patio y porche, terraza de segunda y cubierta plana 29,31 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 29,31 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caras revocadas de muros exteriores y frentes de forjado · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro y +0,68 m² de frente de forjado · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): revoco continuo del IFC (piel vista de la casa, 34 paños de arriba abajo, regla de Enrique del 19 y 21-oct): caras 289,80 m² con los huecos descontados + mochetas y dinteles 18,68 m²; sin medianeras, bajo aleros ni zócalo. Sustituye a la medición por caras de muro (261,81) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): revoco continuo del IFC 20:01: paños de fachada 308,86 m² + cantos de losas y faldones que quedaban vistos 13,43 m² (patinillo, bordes de la cubierta plana, terraza de segunda, faldones sobre la terraza; Enrique 21-oct: el mortero es continuo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paredes 726.4 m² (incluye 27.6 m² de baños y aseos por encima de 2,28 m) y techos sin falso techo 214.4 m² · Opción 2 de cubiertas (16-oct): paredes: +8,09 medianera M2, +5,08 muro M13 (dos caras), −4,72 tabique T2 (dos caras), −1,50 quiebro; techos: −8,52 m² que pasan a falso techo · Opción 3 de cubiertas, IFC final (21-oct): paredes −0,80 m² (cambios de muros de segunda) y techos +8,89 m²: bajo el faldón de la escalera ya no hay falso techo (+8,52) y el faldón a la medianera oeste tiene más superficie en pendiente que la cubierta plana a la que sustituye (+0,37) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +2,84 m² de yeso en paredes (muros de segunda remedidos y trasdosado M13t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caras de baños y aseos con baldosa hasta 2,28 m (por encima, yeso y pintura) · Opción 3 de cubiertas, IFC final (21-oct): +1,06 m² del muro M13b del baño de segunda (hasta 2,28 m). Se mide con la geometría. En el IFC 1843 la baldosa sale en los tabiques de baño (T2, M13b) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): −0,56 m² de baldosa (pared del baño de segunda: muro de carga + trasdosado)</t>
   </si>
   <si>
     <t xml:space="preserve">P2 del BIM (7) + P5 de la Habitación 3, provisional (1)</t>
@@ -3961,10 +3961,10 @@
     <t xml:space="preserve">Mini-balcones de V1, V2 y V3</t>
   </si>
   <si>
-    <t xml:space="preserve">Yeso de paredes y techos más falsos techos · Opción 2 de cubiertas (16-oct): yeso 939,20 + falsos techos 96,96 · Opción 3 de cubiertas, IFC final (21-oct): yeso 947,29 + falsos techos 88,43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Igual que el revoco · Opción 2 de cubiertas (16-oct): igual que el revoco · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): igual que el revoco</t>
+    <t xml:space="preserve">Yeso de paredes y techos más falsos techos · Opción 2 de cubiertas (16-oct): yeso 939,20 + falsos techos 96,96 · Opción 3 de cubiertas, IFC final (21-oct): yeso 947,29 + falsos techos 88,43 · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): yeso 950,13 + falsos techos 88,49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Igual que el revoco · Opción 2 de cubiertas (16-oct): igual que el revoco · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): igual que el revoco · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): igual que el revoco</t>
   </si>
   <si>
     <t xml:space="preserve">Total de las partidas medidas con el BIM</t>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C7/$C$50)</f>
-        <v>0.00248705262373224</v>
+        <v>0.00248239800897721</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C8/$C$50)</f>
-        <v>0.0242458408206481</v>
+        <v>0.02420046379591</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C9/$C$50)</f>
-        <v>0.0251614477307615</v>
+        <v>0.0251143571124336</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C10/$C$50)</f>
-        <v>0.00378328399539629</v>
+        <v>0.0037762034337148</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C14/$C$50)</f>
-        <v>0.00399436515072564</v>
+        <v>0.00398688954253379</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C16/$C$50)</f>
-        <v>0.0131134624351601</v>
+        <v>0.0130889200852484</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C17/$C$50)</f>
-        <v>0.0169124274904269</v>
+        <v>0.0168807752311264</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4816,11 +4816,11 @@
       </c>
       <c r="C18" s="8" t="n">
         <f aca="false">Presupuesto!K286</f>
-        <v>71844.79</v>
+        <v>71882.81</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C18/$C$50)</f>
-        <v>0.187454651144557</v>
+        <v>0.187202837204875</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">SUMIFS(Presupuesto!$K$5:$K$1399,Presupuesto!$M$5:$M$1399,"P",Presupuesto!$O$5:$O$1399,"05.02")</f>
-        <v>50138.3</v>
+        <v>50176.32</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4856,11 +4856,11 @@
       </c>
       <c r="C21" s="8" t="n">
         <f aca="false">Presupuesto!K365</f>
-        <v>56045.68</v>
+        <v>56216.97</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C21/$C$50)</f>
-        <v>0.146232223555243</v>
+        <v>0.146404631135891</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4872,11 +4872,11 @@
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">Presupuesto!K422</f>
-        <v>14344.34</v>
+        <v>14386.83</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C22/$C$50)</f>
-        <v>0.0374266978941537</v>
+        <v>0.0374673081698422</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4888,11 +4888,11 @@
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">Presupuesto!K458</f>
-        <v>7550.42</v>
+        <v>7531.54</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C23/$C$50)</f>
-        <v>0.0197002642376001</v>
+        <v>0.0196142256614899</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4904,11 +4904,11 @@
       </c>
       <c r="C24" s="8" t="n">
         <f aca="false">Presupuesto!K473</f>
-        <v>3673.81</v>
+        <v>3675.43</v>
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C24/$C$50)</f>
-        <v>0.0095855631552599</v>
+        <v>0.00957184233543338</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">Presupuesto!K514</f>
-        <v>21815.11</v>
+        <v>21764.7</v>
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C25/$C$50)</f>
-        <v>0.0569191424281446</v>
+        <v>0.0566813343957052</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4936,11 +4936,11 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">Presupuesto!K545</f>
-        <v>28508.86</v>
+        <v>28920.71</v>
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C26/$C$50)</f>
-        <v>0.0743842163896507</v>
+        <v>0.0753175754534276</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C27/$C$50)</f>
-        <v>0.0275807143419417</v>
+        <v>0.0275290959729916</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C28/$C$50)</f>
-        <v>0.137161030473674</v>
+        <v>0.13690432832344</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C29/$C$50)</f>
-        <v>0.0536864958495679</v>
+        <v>0.0535860195052627</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">Presupuesto!K676</f>
-        <v>8926.64</v>
+        <v>9049.3</v>
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C30/$C$50)</f>
-        <v>0.0232910443066651</v>
+        <v>0.0235668949880796</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C31/$C$50)</f>
-        <v>0.115041029975846</v>
+        <v>0.114825726258325</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C38/$C$50)</f>
-        <v>0.00397766651791838</v>
+        <v>0.00397022216186084</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C41/$C$50)</f>
-        <v>0.00717529815082732</v>
+        <v>0.00716186930403659</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="D42" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C42/$C$50)</f>
-        <v>0.0106860813321</v>
+        <v>0.0106660819193947</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="C48" s="10" t="n">
         <f aca="false">C14+C15+C16+C17+C18+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C38+C41+C42</f>
-        <v>361925.63</v>
+        <v>362644.27</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="C50" s="14" t="n">
         <f aca="false">C11+C48</f>
-        <v>383264.91</v>
+        <v>383983.55</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="C52" s="15" t="n">
         <f aca="false">ROUND(C50*D52,2)</f>
-        <v>19163.25</v>
+        <v>19199.18</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>0.05</v>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="C53" s="15" t="n">
         <f aca="false">ROUND(C50*D53,2)</f>
-        <v>19163.25</v>
+        <v>19199.18</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>0.05</v>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">C50+C52+C53</f>
-        <v>421591.41</v>
+        <v>422381.91</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="C56" s="15" t="n">
         <f aca="false">ROUND(C48*(1+$D$52+$D$53)*D56,2)</f>
-        <v>39811.82</v>
+        <v>39890.87</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>0.1</v>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C57" s="14" t="n">
         <f aca="false">C54+C55+C56</f>
-        <v>466332.6</v>
+        <v>467202.15</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="C61" s="15" t="n">
         <f aca="false">C50/C60</f>
-        <v>1091.36314710405</v>
+        <v>1093.4095050971</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9110,11 +9110,11 @@
       </c>
       <c r="E239" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E8</f>
-        <v>244.74</v>
+        <v>244.03</v>
       </c>
       <c r="H239" s="29" t="n">
         <f aca="false">IF(COUNT(D239:G239)=0,0,D239*IF(E239="",1,E239)*IF(F239="",1,F239)*IF(G239="",1,G239))</f>
-        <v>244.74</v>
+        <v>244.03</v>
       </c>
       <c r="M239" s="23"/>
       <c r="N239" s="23"/>
@@ -9148,14 +9148,14 @@
       <c r="H242" s="30"/>
       <c r="I242" s="31" t="n">
         <f aca="false">ROUND(SUM(H239:H241),2)</f>
-        <v>244.74</v>
+        <v>244.03</v>
       </c>
       <c r="J242" s="32" t="n">
         <v>74</v>
       </c>
       <c r="K242" s="31" t="n">
         <f aca="false">ROUND(I242*J242,2)</f>
-        <v>18110.76</v>
+        <v>18058.22</v>
       </c>
       <c r="L242" s="33" t="s">
         <v>238</v>
@@ -9340,11 +9340,11 @@
       </c>
       <c r="E253" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E10</f>
-        <v>217.97</v>
+        <v>217.99</v>
       </c>
       <c r="H253" s="29" t="n">
         <f aca="false">IF(COUNT(D253:G253)=0,0,D253*IF(E253="",1,E253)*IF(F253="",1,F253)*IF(G253="",1,G253))</f>
-        <v>217.97</v>
+        <v>217.99</v>
       </c>
       <c r="M253" s="23"/>
       <c r="N253" s="23"/>
@@ -9378,14 +9378,14 @@
       <c r="H256" s="30"/>
       <c r="I256" s="31" t="n">
         <f aca="false">ROUND(SUM(H253:H255),2)</f>
-        <v>217.97</v>
+        <v>217.99</v>
       </c>
       <c r="J256" s="32" t="n">
         <v>46</v>
       </c>
       <c r="K256" s="31" t="n">
         <f aca="false">ROUND(I256*J256,2)</f>
-        <v>10026.62</v>
+        <v>10027.54</v>
       </c>
       <c r="L256" s="33" t="s">
         <v>238</v>
@@ -9569,11 +9569,11 @@
       </c>
       <c r="E267" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E11</f>
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="H267" s="29" t="n">
         <f aca="false">IF(COUNT(D267:G267)=0,0,D267*IF(E267="",1,E267)*IF(F267="",1,F267)*IF(G267="",1,G267))</f>
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="M267" s="23"/>
       <c r="N267" s="23"/>
@@ -9583,14 +9583,14 @@
       <c r="H268" s="30"/>
       <c r="I268" s="31" t="n">
         <f aca="false">ROUND(SUM(H267:H267),2)</f>
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="J268" s="32" t="n">
         <v>108</v>
       </c>
       <c r="K268" s="31" t="n">
         <f aca="false">ROUND(I268*J268,2)</f>
-        <v>8772.84</v>
+        <v>8862.48</v>
       </c>
       <c r="L268" s="33" t="s">
         <v>238</v>
@@ -9894,7 +9894,7 @@
       </c>
       <c r="K286" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$285,$M$5:$M$285,"P",$N$5:$N$285,"05")</f>
-        <v>71844.79</v>
+        <v>71882.81</v>
       </c>
       <c r="M286" s="23"/>
       <c r="N286" s="23"/>
@@ -9961,12 +9961,12 @@
       </c>
       <c r="E291" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E14</f>
-        <v>81.09</v>
+        <v>81.61</v>
       </c>
       <c r="G291" s="28"/>
       <c r="H291" s="29" t="n">
         <f aca="false">IF(COUNT(D291:G291)=0,0,D291*IF(E291="",1,E291)*IF(F291="",1,F291)*IF(G291="",1,G291))</f>
-        <v>81.09</v>
+        <v>81.61</v>
       </c>
       <c r="M291" s="23"/>
       <c r="N291" s="23"/>
@@ -10064,14 +10064,14 @@
       <c r="H299" s="30"/>
       <c r="I299" s="31" t="n">
         <f aca="false">ROUND(SUM(H291:H298),2)</f>
-        <v>81.09</v>
+        <v>81.61</v>
       </c>
       <c r="J299" s="32" t="n">
         <v>82</v>
       </c>
       <c r="K299" s="31" t="n">
         <f aca="false">ROUND(I299*J299,2)</f>
-        <v>6649.38</v>
+        <v>6692.02</v>
       </c>
       <c r="L299" s="33" t="s">
         <v>238</v>
@@ -10115,12 +10115,12 @@
       </c>
       <c r="E302" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E15</f>
-        <v>82.91</v>
+        <v>83.8</v>
       </c>
       <c r="G302" s="28"/>
       <c r="H302" s="29" t="n">
         <f aca="false">IF(COUNT(D302:G302)=0,0,D302*IF(E302="",1,E302)*IF(F302="",1,F302)*IF(G302="",1,G302))</f>
-        <v>82.91</v>
+        <v>83.8</v>
       </c>
       <c r="M302" s="23"/>
       <c r="N302" s="23"/>
@@ -10168,14 +10168,14 @@
       <c r="H306" s="30"/>
       <c r="I306" s="31" t="n">
         <f aca="false">ROUND(SUM(H302:H305),2)</f>
-        <v>82.91</v>
+        <v>83.8</v>
       </c>
       <c r="J306" s="32" t="n">
         <v>58</v>
       </c>
       <c r="K306" s="31" t="n">
         <f aca="false">ROUND(I306*J306,2)</f>
-        <v>4808.78</v>
+        <v>4860.4</v>
       </c>
       <c r="L306" s="33" t="s">
         <v>238</v>
@@ -10219,12 +10219,12 @@
       </c>
       <c r="E309" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E16</f>
-        <v>376.13</v>
+        <v>374.64</v>
       </c>
       <c r="G309" s="28"/>
       <c r="H309" s="29" t="n">
         <f aca="false">IF(COUNT(D309:G309)=0,0,D309*IF(E309="",1,E309)*IF(F309="",1,F309)*IF(G309="",1,G309))</f>
-        <v>376.13</v>
+        <v>374.64</v>
       </c>
       <c r="M309" s="23"/>
       <c r="N309" s="23"/>
@@ -10286,14 +10286,14 @@
       <c r="H314" s="30"/>
       <c r="I314" s="31" t="n">
         <f aca="false">ROUND(SUM(H309:H313),2)</f>
-        <v>376.13</v>
+        <v>374.64</v>
       </c>
       <c r="J314" s="32" t="n">
         <v>54</v>
       </c>
       <c r="K314" s="31" t="n">
         <f aca="false">ROUND(I314*J314,2)</f>
-        <v>20311.02</v>
+        <v>20230.56</v>
       </c>
       <c r="L314" s="33" t="s">
         <v>238</v>
@@ -10337,12 +10337,12 @@
       </c>
       <c r="E317" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E17</f>
-        <v>366.97</v>
+        <v>366.74</v>
       </c>
       <c r="G317" s="28"/>
       <c r="H317" s="29" t="n">
         <f aca="false">IF(COUNT(D317:G317)=0,0,D317*IF(E317="",1,E317)*IF(F317="",1,F317)*IF(G317="",1,G317))</f>
-        <v>366.97</v>
+        <v>366.74</v>
       </c>
       <c r="M317" s="23"/>
       <c r="N317" s="23"/>
@@ -10378,14 +10378,14 @@
       <c r="H320" s="30"/>
       <c r="I320" s="31" t="n">
         <f aca="false">ROUND(SUM(H317:H319),2)</f>
-        <v>366.97</v>
+        <v>366.74</v>
       </c>
       <c r="J320" s="32" t="n">
         <v>4.8</v>
       </c>
       <c r="K320" s="31" t="n">
         <f aca="false">ROUND(I320*J320,2)</f>
-        <v>1761.46</v>
+        <v>1760.35</v>
       </c>
       <c r="L320" s="33" t="s">
         <v>238</v>
@@ -10429,12 +10429,12 @@
       </c>
       <c r="E323" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E18</f>
-        <v>95.87</v>
+        <v>99.47</v>
       </c>
       <c r="G323" s="28"/>
       <c r="H323" s="29" t="n">
         <f aca="false">IF(COUNT(D323:G323)=0,0,D323*IF(E323="",1,E323)*IF(F323="",1,F323)*IF(G323="",1,G323))</f>
-        <v>95.87</v>
+        <v>99.47</v>
       </c>
       <c r="M323" s="23"/>
       <c r="N323" s="23"/>
@@ -10470,14 +10470,14 @@
       <c r="H326" s="30"/>
       <c r="I326" s="31" t="n">
         <f aca="false">ROUND(SUM(H323:H325),2)</f>
-        <v>95.87</v>
+        <v>99.47</v>
       </c>
       <c r="J326" s="32" t="n">
         <v>34</v>
       </c>
       <c r="K326" s="31" t="n">
         <f aca="false">ROUND(I326*J326,2)</f>
-        <v>3259.58</v>
+        <v>3381.98</v>
       </c>
       <c r="L326" s="33" t="s">
         <v>238</v>
@@ -10521,12 +10521,12 @@
       </c>
       <c r="E329" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E19</f>
-        <v>110.18</v>
+        <v>111.98</v>
       </c>
       <c r="G329" s="28"/>
       <c r="H329" s="29" t="n">
         <f aca="false">IF(COUNT(D329:G329)=0,0,D329*IF(E329="",1,E329)*IF(F329="",1,F329)*IF(G329="",1,G329))</f>
-        <v>110.18</v>
+        <v>111.98</v>
       </c>
       <c r="M329" s="23"/>
       <c r="N329" s="23"/>
@@ -10562,14 +10562,14 @@
       <c r="H332" s="30"/>
       <c r="I332" s="31" t="n">
         <f aca="false">ROUND(SUM(H329:H331),2)</f>
-        <v>110.18</v>
+        <v>111.98</v>
       </c>
       <c r="J332" s="32" t="n">
         <v>33</v>
       </c>
       <c r="K332" s="31" t="n">
         <f aca="false">ROUND(I332*J332,2)</f>
-        <v>3635.94</v>
+        <v>3695.34</v>
       </c>
       <c r="L332" s="33" t="s">
         <v>238</v>
@@ -10731,11 +10731,11 @@
       </c>
       <c r="E342" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E20</f>
-        <v>44.58</v>
+        <v>43.78</v>
       </c>
       <c r="H342" s="29" t="n">
         <f aca="false">IF(COUNT(D342:G342)=0,0,D342*IF(E342="",1,E342)*IF(F342="",1,F342)*IF(G342="",1,G342))</f>
-        <v>44.58</v>
+        <v>43.78</v>
       </c>
       <c r="M342" s="23"/>
       <c r="N342" s="23"/>
@@ -10757,14 +10757,14 @@
       <c r="H344" s="30"/>
       <c r="I344" s="31" t="n">
         <f aca="false">ROUND(SUM(H342:H343),2)</f>
-        <v>44.58</v>
+        <v>43.78</v>
       </c>
       <c r="J344" s="32" t="n">
         <v>29</v>
       </c>
       <c r="K344" s="31" t="n">
         <f aca="false">ROUND(I344*J344,2)</f>
-        <v>1292.82</v>
+        <v>1269.62</v>
       </c>
       <c r="L344" s="33" t="s">
         <v>238</v>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="K365" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$364,$M$5:$M$364,"P",$N$5:$N$364,"06")</f>
-        <v>56045.68</v>
+        <v>56216.97</v>
       </c>
       <c r="M365" s="23"/>
       <c r="N365" s="23"/>
@@ -11155,11 +11155,11 @@
       </c>
       <c r="E370" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E21</f>
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="H370" s="29" t="n">
         <f aca="false">IF(COUNT(D370:G370)=0,0,D370*IF(E370="",1,E370)*IF(F370="",1,F370)*IF(G370="",1,G370))</f>
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="M370" s="23"/>
       <c r="N370" s="23"/>
@@ -11169,14 +11169,14 @@
       <c r="H371" s="30"/>
       <c r="I371" s="31" t="n">
         <f aca="false">ROUND(SUM(H370:H370),2)</f>
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="J371" s="32" t="n">
         <v>17.5</v>
       </c>
       <c r="K371" s="31" t="n">
         <f aca="false">ROUND(I371*J371,2)</f>
-        <v>1421.53</v>
+        <v>1436.05</v>
       </c>
       <c r="L371" s="33" t="s">
         <v>238</v>
@@ -11220,11 +11220,11 @@
       </c>
       <c r="E374" s="28" t="n">
         <f aca="false">'Mediciones BIM'!E22</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="H374" s="29" t="n">
         <f aca="false">IF(COUNT(D374:G374)=0,0,D374*IF(E374="",1,E374)*IF(F374="",1,F374)*IF(G374="",1,G374))</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="M374" s="23"/>
       <c r="N374" s="23"/>
@@ -11234,14 +11234,14 @@
       <c r="H375" s="30"/>
       <c r="I375" s="31" t="n">
         <f aca="false">ROUND(SUM(H374:H374),2)</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="J375" s="32" t="n">
         <v>19.5</v>
       </c>
       <c r="K375" s="31" t="n">
         <f aca="false">ROUND(I375*J375,2)</f>
-        <v>1707.03</v>
+        <v>1723.22</v>
       </c>
       <c r="L375" s="33" t="s">
         <v>238</v>
@@ -11285,11 +11285,11 @@
       </c>
       <c r="E378" s="28" t="n">
         <f aca="false">'Mediciones BIM'!E22</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="H378" s="29" t="n">
         <f aca="false">IF(COUNT(D378:G378)=0,0,D378*IF(E378="",1,E378)*IF(F378="",1,F378)*IF(G378="",1,G378))</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="M378" s="23"/>
       <c r="N378" s="23"/>
@@ -11299,14 +11299,14 @@
       <c r="H379" s="30"/>
       <c r="I379" s="31" t="n">
         <f aca="false">ROUND(SUM(H378:H378),2)</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="J379" s="32" t="n">
         <v>3.9</v>
       </c>
       <c r="K379" s="31" t="n">
         <f aca="false">ROUND(I379*J379,2)</f>
-        <v>341.41</v>
+        <v>344.64</v>
       </c>
       <c r="L379" s="33" t="s">
         <v>212</v>
@@ -11350,11 +11350,11 @@
       </c>
       <c r="E382" s="28" t="n">
         <f aca="false">'Mediciones BIM'!E22</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="H382" s="29" t="n">
         <f aca="false">IF(COUNT(D382:G382)=0,0,D382*IF(E382="",1,E382)*IF(F382="",1,F382)*IF(G382="",1,G382))</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="M382" s="23"/>
       <c r="N382" s="23"/>
@@ -11364,14 +11364,14 @@
       <c r="H383" s="30"/>
       <c r="I383" s="31" t="n">
         <f aca="false">ROUND(SUM(H382:H382),2)</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="J383" s="32" t="n">
         <v>9.5</v>
       </c>
       <c r="K383" s="31" t="n">
         <f aca="false">ROUND(I383*J383,2)</f>
-        <v>831.63</v>
+        <v>839.52</v>
       </c>
       <c r="L383" s="33" t="s">
         <v>238</v>
@@ -11415,11 +11415,11 @@
       </c>
       <c r="E386" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E22</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="H386" s="29" t="n">
         <f aca="false">IF(COUNT(D386:G386)=0,0,D386*IF(E386="",1,E386)*IF(F386="",1,F386)*IF(G386="",1,G386))</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="M386" s="23"/>
       <c r="N386" s="23"/>
@@ -11429,14 +11429,14 @@
       <c r="H387" s="30"/>
       <c r="I387" s="31" t="n">
         <f aca="false">ROUND(SUM(H386:H386),2)</f>
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="J387" s="32" t="n">
         <v>36.12</v>
       </c>
       <c r="K387" s="31" t="n">
         <f aca="false">ROUND(I387*J387,2)</f>
-        <v>3161.94</v>
+        <v>3191.92</v>
       </c>
       <c r="L387" s="33" t="s">
         <v>212</v>
@@ -11708,11 +11708,11 @@
       </c>
       <c r="E404" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E23</f>
-        <v>30.02</v>
+        <v>29.31</v>
       </c>
       <c r="H404" s="29" t="n">
         <f aca="false">IF(COUNT(D404:G404)=0,0,D404*IF(E404="",1,E404)*IF(F404="",1,F404)*IF(G404="",1,G404))</f>
-        <v>30.02</v>
+        <v>29.31</v>
       </c>
       <c r="M404" s="23"/>
       <c r="N404" s="23"/>
@@ -11722,14 +11722,14 @@
       <c r="H405" s="30"/>
       <c r="I405" s="31" t="n">
         <f aca="false">ROUND(SUM(H404:H404),2)</f>
-        <v>30.02</v>
+        <v>29.31</v>
       </c>
       <c r="J405" s="32" t="n">
         <v>24.5</v>
       </c>
       <c r="K405" s="31" t="n">
         <f aca="false">ROUND(I405*J405,2)</f>
-        <v>735.49</v>
+        <v>718.1</v>
       </c>
       <c r="L405" s="33" t="s">
         <v>438</v>
@@ -11895,11 +11895,11 @@
       </c>
       <c r="E416" s="36" t="n">
         <f aca="false">'Mediciones BIM'!E24</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="H416" s="29" t="n">
         <f aca="false">IF(COUNT(D416:G416)=0,0,D416*IF(E416="",1,E416)*IF(F416="",1,F416)*IF(G416="",1,G416))</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="M416" s="23"/>
       <c r="N416" s="23"/>
@@ -11909,14 +11909,14 @@
       <c r="H417" s="30"/>
       <c r="I417" s="31" t="n">
         <f aca="false">ROUND(SUM(H416:H416),2)</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="J417" s="32" t="n">
         <v>13</v>
       </c>
       <c r="K417" s="31" t="n">
         <f aca="false">ROUND(I417*J417,2)</f>
-        <v>919.36</v>
+        <v>910.13</v>
       </c>
       <c r="L417" s="33" t="s">
         <v>238</v>
@@ -11960,11 +11960,11 @@
       </c>
       <c r="E420" s="36" t="n">
         <f aca="false">'Mediciones BIM'!E25</f>
-        <v>59.67</v>
+        <v>58.96</v>
       </c>
       <c r="H420" s="29" t="n">
         <f aca="false">IF(COUNT(D420:G420)=0,0,D420*IF(E420="",1,E420)*IF(F420="",1,F420)*IF(G420="",1,G420))</f>
-        <v>59.67</v>
+        <v>58.96</v>
       </c>
       <c r="M420" s="23"/>
       <c r="N420" s="23"/>
@@ -11974,14 +11974,14 @@
       <c r="H421" s="30"/>
       <c r="I421" s="31" t="n">
         <f aca="false">ROUND(SUM(H420:H420),2)</f>
-        <v>59.67</v>
+        <v>58.96</v>
       </c>
       <c r="J421" s="32" t="n">
         <v>3.8</v>
       </c>
       <c r="K421" s="31" t="n">
         <f aca="false">ROUND(I421*J421,2)</f>
-        <v>226.75</v>
+        <v>224.05</v>
       </c>
       <c r="L421" s="33" t="s">
         <v>238</v>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="K422" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$421,$M$5:$M$421,"P",$N$5:$N$421,"07")</f>
-        <v>14344.34</v>
+        <v>14386.83</v>
       </c>
       <c r="M422" s="23"/>
       <c r="N422" s="23"/>
@@ -12209,11 +12209,11 @@
       </c>
       <c r="E436" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E28</f>
-        <v>221.12</v>
+        <v>220.41</v>
       </c>
       <c r="H436" s="29" t="n">
         <f aca="false">IF(COUNT(D436:G436)=0,0,D436*IF(E436="",1,E436)*IF(F436="",1,F436)*IF(G436="",1,G436))</f>
-        <v>221.12</v>
+        <v>220.41</v>
       </c>
       <c r="M436" s="23"/>
       <c r="N436" s="23"/>
@@ -12223,14 +12223,14 @@
       <c r="H437" s="30"/>
       <c r="I437" s="31" t="n">
         <f aca="false">ROUND(SUM(H436:H436),2)</f>
-        <v>221.12</v>
+        <v>220.41</v>
       </c>
       <c r="J437" s="32" t="n">
         <v>4.6</v>
       </c>
       <c r="K437" s="31" t="n">
         <f aca="false">ROUND(I437*J437,2)</f>
-        <v>1017.15</v>
+        <v>1013.89</v>
       </c>
       <c r="L437" s="33" t="s">
         <v>238</v>
@@ -12530,11 +12530,11 @@
       </c>
       <c r="E456" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E29</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="H456" s="29" t="n">
         <f aca="false">IF(COUNT(D456:G456)=0,0,D456*IF(E456="",1,E456)*IF(F456="",1,F456)*IF(G456="",1,G456))</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="M456" s="23"/>
       <c r="N456" s="23"/>
@@ -12544,14 +12544,14 @@
       <c r="H457" s="30"/>
       <c r="I457" s="31" t="n">
         <f aca="false">ROUND(SUM(H456:H456),2)</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="J457" s="32" t="n">
         <v>22</v>
       </c>
       <c r="K457" s="31" t="n">
         <f aca="false">ROUND(I457*J457,2)</f>
-        <v>1555.84</v>
+        <v>1540.22</v>
       </c>
       <c r="L457" s="33" t="s">
         <v>238</v>
@@ -12570,7 +12570,7 @@
       </c>
       <c r="K458" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$457,$M$5:$M$457,"P",$N$5:$N$457,"08")</f>
-        <v>7550.42</v>
+        <v>7531.54</v>
       </c>
       <c r="M458" s="23"/>
       <c r="N458" s="23"/>
@@ -12637,11 +12637,11 @@
       </c>
       <c r="E463" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E30</f>
-        <v>88.43</v>
+        <v>88.49</v>
       </c>
       <c r="H463" s="29" t="n">
         <f aca="false">IF(COUNT(D463:G463)=0,0,D463*IF(E463="",1,E463)*IF(F463="",1,F463)*IF(G463="",1,G463))</f>
-        <v>88.43</v>
+        <v>88.49</v>
       </c>
       <c r="M463" s="23"/>
       <c r="N463" s="23"/>
@@ -12651,14 +12651,14 @@
       <c r="H464" s="30"/>
       <c r="I464" s="31" t="n">
         <f aca="false">ROUND(SUM(H463:H463),2)</f>
-        <v>88.43</v>
+        <v>88.49</v>
       </c>
       <c r="J464" s="32" t="n">
         <v>27</v>
       </c>
       <c r="K464" s="31" t="n">
         <f aca="false">ROUND(I464*J464,2)</f>
-        <v>2387.61</v>
+        <v>2389.23</v>
       </c>
       <c r="L464" s="33" t="s">
         <v>238</v>
@@ -12803,7 +12803,7 @@
       </c>
       <c r="K473" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$472,$M$5:$M$472,"P",$N$5:$N$472,"09")</f>
-        <v>3673.81</v>
+        <v>3675.43</v>
       </c>
       <c r="M473" s="23"/>
       <c r="N473" s="23"/>
@@ -13076,11 +13076,11 @@
       </c>
       <c r="E491" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E34</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="H491" s="29" t="n">
         <f aca="false">IF(COUNT(D491:G491)=0,0,D491*IF(E491="",1,E491)*IF(F491="",1,F491)*IF(G491="",1,G491))</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="M491" s="23"/>
       <c r="N491" s="23"/>
@@ -13102,14 +13102,14 @@
       <c r="H493" s="30"/>
       <c r="I493" s="31" t="n">
         <f aca="false">ROUND(SUM(H491:H492),2)</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="J493" s="32" t="n">
         <v>56</v>
       </c>
       <c r="K493" s="31" t="n">
         <f aca="false">ROUND(I493*J493,2)</f>
-        <v>3960.32</v>
+        <v>3920.56</v>
       </c>
       <c r="L493" s="33" t="s">
         <v>238</v>
@@ -13408,11 +13408,11 @@
       </c>
       <c r="E512" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E37</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="H512" s="29" t="n">
         <f aca="false">IF(COUNT(D512:G512)=0,0,D512*IF(E512="",1,E512)*IF(F512="",1,F512)*IF(G512="",1,G512))</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="M512" s="23"/>
       <c r="N512" s="23"/>
@@ -13422,14 +13422,14 @@
       <c r="H513" s="30"/>
       <c r="I513" s="31" t="n">
         <f aca="false">ROUND(SUM(H512:H512),2)</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="J513" s="32" t="n">
         <v>15</v>
       </c>
       <c r="K513" s="31" t="n">
         <f aca="false">ROUND(I513*J513,2)</f>
-        <v>1060.8</v>
+        <v>1050.15</v>
       </c>
       <c r="L513" s="33" t="s">
         <v>523</v>
@@ -13448,7 +13448,7 @@
       </c>
       <c r="K514" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$513,$M$5:$M$513,"P",$N$5:$N$513,"10")</f>
-        <v>21815.11</v>
+        <v>21764.7</v>
       </c>
       <c r="M514" s="23"/>
       <c r="N514" s="23"/>
@@ -13515,11 +13515,11 @@
       </c>
       <c r="E519" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E38</f>
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="H519" s="29" t="n">
         <f aca="false">IF(COUNT(D519:G519)=0,0,D519*IF(E519="",1,E519)*IF(F519="",1,F519)*IF(G519="",1,G519))</f>
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="M519" s="23"/>
       <c r="N519" s="23"/>
@@ -13553,14 +13553,14 @@
       <c r="H522" s="30"/>
       <c r="I522" s="31" t="n">
         <f aca="false">ROUND(SUM(H519:H521),2)</f>
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="J522" s="32" t="n">
         <v>29.56</v>
       </c>
       <c r="K522" s="31" t="n">
         <f aca="false">ROUND(I522*J522,2)</f>
-        <v>9118.96</v>
+        <v>9526.89</v>
       </c>
       <c r="L522" s="33" t="s">
         <v>212</v>
@@ -13604,11 +13604,11 @@
       </c>
       <c r="E525" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E39</f>
-        <v>947.29</v>
+        <v>950.13</v>
       </c>
       <c r="H525" s="29" t="n">
         <f aca="false">IF(COUNT(D525:G525)=0,0,D525*IF(E525="",1,E525)*IF(F525="",1,F525)*IF(G525="",1,G525))</f>
-        <v>947.29</v>
+        <v>950.13</v>
       </c>
       <c r="M525" s="23"/>
       <c r="N525" s="23"/>
@@ -13690,14 +13690,14 @@
       <c r="H532" s="30"/>
       <c r="I532" s="31" t="n">
         <f aca="false">ROUND(SUM(H525:H531),2)</f>
-        <v>947.29</v>
+        <v>950.13</v>
       </c>
       <c r="J532" s="32" t="n">
         <v>14</v>
       </c>
       <c r="K532" s="31" t="n">
         <f aca="false">ROUND(I532*J532,2)</f>
-        <v>13262.06</v>
+        <v>13301.82</v>
       </c>
       <c r="L532" s="33" t="s">
         <v>238</v>
@@ -13741,12 +13741,12 @@
       </c>
       <c r="E535" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E40</f>
-        <v>88.58</v>
+        <v>88.02</v>
       </c>
       <c r="G535" s="28"/>
       <c r="H535" s="29" t="n">
         <f aca="false">IF(COUNT(D535:G535)=0,0,D535*IF(E535="",1,E535)*IF(F535="",1,F535)*IF(G535="",1,G535))</f>
-        <v>88.58</v>
+        <v>88.02</v>
       </c>
       <c r="M535" s="23"/>
       <c r="N535" s="23"/>
@@ -13808,14 +13808,14 @@
       <c r="H540" s="30"/>
       <c r="I540" s="31" t="n">
         <f aca="false">ROUND(SUM(H535:H539),2)</f>
-        <v>88.58</v>
+        <v>88.02</v>
       </c>
       <c r="J540" s="32" t="n">
         <v>64</v>
       </c>
       <c r="K540" s="31" t="n">
         <f aca="false">ROUND(I540*J540,2)</f>
-        <v>5669.12</v>
+        <v>5633.28</v>
       </c>
       <c r="L540" s="33" t="s">
         <v>238</v>
@@ -13898,7 +13898,7 @@
       </c>
       <c r="K545" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$544,$M$5:$M$544,"P",$N$5:$N$544,"11")</f>
-        <v>28508.86</v>
+        <v>28920.71</v>
       </c>
       <c r="M545" s="23"/>
       <c r="N545" s="23"/>
@@ -15841,11 +15841,11 @@
       </c>
       <c r="E669" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E57</f>
-        <v>1035.72</v>
+        <v>1038.62</v>
       </c>
       <c r="H669" s="29" t="n">
         <f aca="false">IF(COUNT(D669:G669)=0,0,D669*IF(E669="",1,E669)*IF(F669="",1,F669)*IF(G669="",1,G669))</f>
-        <v>1035.72</v>
+        <v>1038.62</v>
       </c>
       <c r="M669" s="23"/>
       <c r="N669" s="23"/>
@@ -15867,14 +15867,14 @@
       <c r="H671" s="30"/>
       <c r="I671" s="31" t="n">
         <f aca="false">ROUND(SUM(H669:H670),2)</f>
-        <v>1035.72</v>
+        <v>1038.62</v>
       </c>
       <c r="J671" s="32" t="n">
         <v>6.37</v>
       </c>
       <c r="K671" s="31" t="n">
         <f aca="false">ROUND(I671*J671,2)</f>
-        <v>6597.54</v>
+        <v>6616.01</v>
       </c>
       <c r="L671" s="33" t="s">
         <v>212</v>
@@ -15918,11 +15918,11 @@
       </c>
       <c r="E674" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E58</f>
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="H674" s="29" t="n">
         <f aca="false">IF(COUNT(D674:G674)=0,0,D674*IF(E674="",1,E674)*IF(F674="",1,F674)*IF(G674="",1,G674))</f>
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="M674" s="23"/>
       <c r="N674" s="23"/>
@@ -15932,14 +15932,14 @@
       <c r="H675" s="30"/>
       <c r="I675" s="31" t="n">
         <f aca="false">ROUND(SUM(H674:H674),2)</f>
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="J675" s="32" t="n">
         <v>7.55</v>
       </c>
       <c r="K675" s="31" t="n">
         <f aca="false">ROUND(I675*J675,2)</f>
-        <v>2329.1</v>
+        <v>2433.29</v>
       </c>
       <c r="L675" s="33" t="s">
         <v>212</v>
@@ -15958,7 +15958,7 @@
       </c>
       <c r="K676" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$675,$M$5:$M$675,"P",$N$5:$N$675,"15")</f>
-        <v>8926.64</v>
+        <v>9049.3</v>
       </c>
       <c r="M676" s="23"/>
       <c r="N676" s="23"/>
@@ -27626,15 +27626,15 @@
         <v>238</v>
       </c>
       <c r="E8" s="42" t="n">
-        <v>244.74</v>
+        <v>244.03</v>
       </c>
       <c r="F8" s="29" t="n">
         <f aca="false">E8-D8</f>
-        <v>6.74000000000001</v>
+        <v>6.03</v>
       </c>
       <c r="G8" s="43" t="n">
         <f aca="false">IF(D8=0,"-",F8/D8)</f>
-        <v>0.0283193277310925</v>
+        <v>0.0253361344537815</v>
       </c>
       <c r="H8" s="44" t="n">
         <f aca="false">Presupuesto!J242</f>
@@ -27646,11 +27646,11 @@
       </c>
       <c r="J8" s="44" t="n">
         <f aca="false">Presupuesto!K242</f>
-        <v>18110.76</v>
+        <v>18058.22</v>
       </c>
       <c r="K8" s="29" t="n">
         <f aca="false">J8-I8</f>
-        <v>498.759999999998</v>
+        <v>446.220000000001</v>
       </c>
       <c r="L8" s="26" t="s">
         <v>1266</v>
@@ -27720,15 +27720,15 @@
         <v>198</v>
       </c>
       <c r="E10" s="42" t="n">
-        <v>217.97</v>
+        <v>217.99</v>
       </c>
       <c r="F10" s="29" t="n">
         <f aca="false">E10-D10</f>
-        <v>19.97</v>
+        <v>19.99</v>
       </c>
       <c r="G10" s="43" t="n">
         <f aca="false">IF(D10=0,"-",F10/D10)</f>
-        <v>0.100858585858586</v>
+        <v>0.100959595959596</v>
       </c>
       <c r="H10" s="44" t="n">
         <f aca="false">Presupuesto!J256</f>
@@ -27740,11 +27740,11 @@
       </c>
       <c r="J10" s="44" t="n">
         <f aca="false">Presupuesto!K256</f>
-        <v>10026.62</v>
+        <v>10027.54</v>
       </c>
       <c r="K10" s="29" t="n">
         <f aca="false">J10-I10</f>
-        <v>918.620000000001</v>
+        <v>919.540000000001</v>
       </c>
       <c r="L10" s="26" t="s">
         <v>1268</v>
@@ -27767,15 +27767,15 @@
         <v>70</v>
       </c>
       <c r="E11" s="42" t="n">
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="F11" s="29" t="n">
         <f aca="false">E11-D11</f>
-        <v>11.23</v>
+        <v>12.06</v>
       </c>
       <c r="G11" s="43" t="n">
         <f aca="false">IF(D11=0,"-",F11/D11)</f>
-        <v>0.160428571428571</v>
+        <v>0.172285714285714</v>
       </c>
       <c r="H11" s="44" t="n">
         <f aca="false">Presupuesto!J268</f>
@@ -27787,11 +27787,11 @@
       </c>
       <c r="J11" s="44" t="n">
         <f aca="false">Presupuesto!K268</f>
-        <v>8772.84</v>
+        <v>8862.48</v>
       </c>
       <c r="K11" s="29" t="n">
         <f aca="false">J11-I11</f>
-        <v>1212.84</v>
+        <v>1302.48</v>
       </c>
       <c r="L11" s="26" t="s">
         <v>1269</v>
@@ -27908,15 +27908,15 @@
         <v>85.85</v>
       </c>
       <c r="E14" s="42" t="n">
-        <v>81.09</v>
+        <v>81.61</v>
       </c>
       <c r="F14" s="29" t="n">
         <f aca="false">E14-D14</f>
-        <v>-4.75999999999999</v>
+        <v>-4.24</v>
       </c>
       <c r="G14" s="43" t="n">
         <f aca="false">IF(D14=0,"-",F14/D14)</f>
-        <v>-0.0554455445544553</v>
+        <v>-0.0493884682585905</v>
       </c>
       <c r="H14" s="44" t="n">
         <f aca="false">Presupuesto!J299</f>
@@ -27928,11 +27928,11 @@
       </c>
       <c r="J14" s="44" t="n">
         <f aca="false">Presupuesto!K299</f>
-        <v>6649.38</v>
+        <v>6692.02</v>
       </c>
       <c r="K14" s="29" t="n">
         <f aca="false">J14-I14</f>
-        <v>-390.32</v>
+        <v>-347.679999999999</v>
       </c>
       <c r="L14" s="26" t="s">
         <v>1272</v>
@@ -27955,15 +27955,15 @@
         <v>70.54</v>
       </c>
       <c r="E15" s="42" t="n">
-        <v>82.91</v>
+        <v>83.8</v>
       </c>
       <c r="F15" s="29" t="n">
         <f aca="false">E15-D15</f>
-        <v>12.37</v>
+        <v>13.26</v>
       </c>
       <c r="G15" s="43" t="n">
         <f aca="false">IF(D15=0,"-",F15/D15)</f>
-        <v>0.175361497022966</v>
+        <v>0.18797845194216</v>
       </c>
       <c r="H15" s="44" t="n">
         <f aca="false">Presupuesto!J306</f>
@@ -27975,11 +27975,11 @@
       </c>
       <c r="J15" s="44" t="n">
         <f aca="false">Presupuesto!K306</f>
-        <v>4808.78</v>
+        <v>4860.4</v>
       </c>
       <c r="K15" s="29" t="n">
         <f aca="false">J15-I15</f>
-        <v>717.46</v>
+        <v>769.08</v>
       </c>
       <c r="L15" s="26" t="s">
         <v>1273</v>
@@ -28002,15 +28002,15 @@
         <v>327.98</v>
       </c>
       <c r="E16" s="42" t="n">
-        <v>376.13</v>
+        <v>374.64</v>
       </c>
       <c r="F16" s="29" t="n">
         <f aca="false">E16-D16</f>
-        <v>48.15</v>
+        <v>46.66</v>
       </c>
       <c r="G16" s="43" t="n">
         <f aca="false">IF(D16=0,"-",F16/D16)</f>
-        <v>0.146807732178791</v>
+        <v>0.14226477224221</v>
       </c>
       <c r="H16" s="44" t="n">
         <f aca="false">Presupuesto!J314</f>
@@ -28022,11 +28022,11 @@
       </c>
       <c r="J16" s="44" t="n">
         <f aca="false">Presupuesto!K314</f>
-        <v>20311.02</v>
+        <v>20230.56</v>
       </c>
       <c r="K16" s="29" t="n">
         <f aca="false">J16-I16</f>
-        <v>2600.1</v>
+        <v>2519.64</v>
       </c>
       <c r="L16" s="26" t="s">
         <v>1274</v>
@@ -28049,15 +28049,15 @@
         <v>350.03</v>
       </c>
       <c r="E17" s="42" t="n">
-        <v>366.97</v>
+        <v>366.74</v>
       </c>
       <c r="F17" s="29" t="n">
         <f aca="false">E17-D17</f>
-        <v>16.9400000000001</v>
+        <v>16.71</v>
       </c>
       <c r="G17" s="43" t="n">
         <f aca="false">IF(D17=0,"-",F17/D17)</f>
-        <v>0.048395851784133</v>
+        <v>0.0477387652486931</v>
       </c>
       <c r="H17" s="44" t="n">
         <f aca="false">Presupuesto!J320</f>
@@ -28069,11 +28069,11 @@
       </c>
       <c r="J17" s="44" t="n">
         <f aca="false">Presupuesto!K320</f>
-        <v>1761.46</v>
+        <v>1760.35</v>
       </c>
       <c r="K17" s="29" t="n">
         <f aca="false">J17-I17</f>
-        <v>81.3199999999999</v>
+        <v>80.2099999999998</v>
       </c>
       <c r="L17" s="26" t="s">
         <v>1275</v>
@@ -28096,15 +28096,15 @@
         <v>83.01</v>
       </c>
       <c r="E18" s="42" t="n">
-        <v>95.87</v>
+        <v>99.47</v>
       </c>
       <c r="F18" s="29" t="n">
         <f aca="false">E18-D18</f>
-        <v>12.86</v>
+        <v>16.46</v>
       </c>
       <c r="G18" s="43" t="n">
         <f aca="false">IF(D18=0,"-",F18/D18)</f>
-        <v>0.154921093844115</v>
+        <v>0.198289362727382</v>
       </c>
       <c r="H18" s="44" t="n">
         <f aca="false">Presupuesto!J326</f>
@@ -28116,11 +28116,11 @@
       </c>
       <c r="J18" s="44" t="n">
         <f aca="false">Presupuesto!K326</f>
-        <v>3259.58</v>
+        <v>3381.98</v>
       </c>
       <c r="K18" s="29" t="n">
         <f aca="false">J18-I18</f>
-        <v>437.24</v>
+        <v>559.64</v>
       </c>
       <c r="L18" s="26" t="s">
         <v>1276</v>
@@ -28143,15 +28143,15 @@
         <v>77.47</v>
       </c>
       <c r="E19" s="42" t="n">
-        <v>110.18</v>
+        <v>111.98</v>
       </c>
       <c r="F19" s="29" t="n">
         <f aca="false">E19-D19</f>
-        <v>32.71</v>
+        <v>34.51</v>
       </c>
       <c r="G19" s="43" t="n">
         <f aca="false">IF(D19=0,"-",F19/D19)</f>
-        <v>0.422227959210017</v>
+        <v>0.445462759777979</v>
       </c>
       <c r="H19" s="44" t="n">
         <f aca="false">Presupuesto!J332</f>
@@ -28163,11 +28163,11 @@
       </c>
       <c r="J19" s="44" t="n">
         <f aca="false">Presupuesto!K332</f>
-        <v>3635.94</v>
+        <v>3695.34</v>
       </c>
       <c r="K19" s="29" t="n">
         <f aca="false">J19-I19</f>
-        <v>1079.43</v>
+        <v>1138.83</v>
       </c>
       <c r="L19" s="26" t="s">
         <v>1277</v>
@@ -28190,15 +28190,15 @@
         <v>62.72</v>
       </c>
       <c r="E20" s="42" t="n">
-        <v>44.58</v>
+        <v>43.78</v>
       </c>
       <c r="F20" s="29" t="n">
         <f aca="false">E20-D20</f>
-        <v>-18.14</v>
+        <v>-18.94</v>
       </c>
       <c r="G20" s="43" t="n">
         <f aca="false">IF(D20=0,"-",F20/D20)</f>
-        <v>-0.28922193877551</v>
+        <v>-0.301977040816327</v>
       </c>
       <c r="H20" s="44" t="n">
         <f aca="false">Presupuesto!J344</f>
@@ -28210,11 +28210,11 @@
       </c>
       <c r="J20" s="44" t="n">
         <f aca="false">Presupuesto!K344</f>
-        <v>1292.82</v>
+        <v>1269.62</v>
       </c>
       <c r="K20" s="29" t="n">
         <f aca="false">J20-I20</f>
-        <v>-526.06</v>
+        <v>-549.26</v>
       </c>
       <c r="L20" s="26" t="s">
         <v>1278</v>
@@ -28237,15 +28237,15 @@
         <v>70</v>
       </c>
       <c r="E21" s="42" t="n">
-        <v>81.23</v>
+        <v>82.06</v>
       </c>
       <c r="F21" s="29" t="n">
         <f aca="false">E21-D21</f>
-        <v>11.23</v>
+        <v>12.06</v>
       </c>
       <c r="G21" s="43" t="n">
         <f aca="false">IF(D21=0,"-",F21/D21)</f>
-        <v>0.160428571428571</v>
+        <v>0.172285714285714</v>
       </c>
       <c r="H21" s="44" t="n">
         <f aca="false">Presupuesto!J371</f>
@@ -28257,11 +28257,11 @@
       </c>
       <c r="J21" s="44" t="n">
         <f aca="false">Presupuesto!K371</f>
-        <v>1421.53</v>
+        <v>1436.05</v>
       </c>
       <c r="K21" s="29" t="n">
         <f aca="false">J21-I21</f>
-        <v>196.53</v>
+        <v>211.05</v>
       </c>
       <c r="L21" s="26" t="s">
         <v>1279</v>
@@ -28284,15 +28284,15 @@
         <v>70</v>
       </c>
       <c r="E22" s="42" t="n">
-        <v>87.54</v>
+        <v>88.37</v>
       </c>
       <c r="F22" s="29" t="n">
         <f aca="false">E22-D22</f>
-        <v>17.54</v>
+        <v>18.37</v>
       </c>
       <c r="G22" s="43" t="n">
         <f aca="false">IF(D22=0,"-",F22/D22)</f>
-        <v>0.250571428571429</v>
+        <v>0.262428571428572</v>
       </c>
       <c r="H22" s="44" t="n">
         <f aca="false">Presupuesto!J387</f>
@@ -28304,11 +28304,11 @@
       </c>
       <c r="J22" s="44" t="n">
         <f aca="false">Presupuesto!K387</f>
-        <v>3161.94</v>
+        <v>3191.92</v>
       </c>
       <c r="K22" s="29" t="n">
         <f aca="false">J22-I22</f>
-        <v>633.54</v>
+        <v>663.52</v>
       </c>
       <c r="L22" s="26" t="s">
         <v>1280</v>
@@ -28331,15 +28331,15 @@
         <v>77.3</v>
       </c>
       <c r="E23" s="42" t="n">
-        <v>30.02</v>
+        <v>29.31</v>
       </c>
       <c r="F23" s="29" t="n">
         <f aca="false">E23-D23</f>
-        <v>-47.28</v>
+        <v>-47.99</v>
       </c>
       <c r="G23" s="43" t="n">
         <f aca="false">IF(D23=0,"-",F23/D23)</f>
-        <v>-0.611642949547219</v>
+        <v>-0.620827943078913</v>
       </c>
       <c r="H23" s="44" t="n">
         <f aca="false">Presupuesto!J405</f>
@@ -28350,11 +28350,11 @@
       </c>
       <c r="J23" s="44" t="n">
         <f aca="false">Presupuesto!K405</f>
-        <v>735.49</v>
+        <v>718.1</v>
       </c>
       <c r="K23" s="29" t="n">
         <f aca="false">J23-I23</f>
-        <v>-4984.71</v>
+        <v>-5002.1</v>
       </c>
       <c r="L23" s="26" t="s">
         <v>1281</v>
@@ -28377,11 +28377,11 @@
         <v>0</v>
       </c>
       <c r="E24" s="42" t="n">
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="F24" s="29" t="n">
         <f aca="false">E24-D24</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="G24" s="43" t="str">
         <f aca="false">IF(D24=0,"-",F24/D24)</f>
@@ -28397,11 +28397,11 @@
       </c>
       <c r="J24" s="44" t="n">
         <f aca="false">Presupuesto!K417</f>
-        <v>919.36</v>
+        <v>910.13</v>
       </c>
       <c r="K24" s="29" t="n">
         <f aca="false">J24-I24</f>
-        <v>919.36</v>
+        <v>910.13</v>
       </c>
       <c r="L24" s="26" t="s">
         <v>1282</v>
@@ -28424,11 +28424,11 @@
         <v>0</v>
       </c>
       <c r="E25" s="42" t="n">
-        <v>59.67</v>
+        <v>58.96</v>
       </c>
       <c r="F25" s="29" t="n">
         <f aca="false">E25-D25</f>
-        <v>59.67</v>
+        <v>58.96</v>
       </c>
       <c r="G25" s="43" t="str">
         <f aca="false">IF(D25=0,"-",F25/D25)</f>
@@ -28444,11 +28444,11 @@
       </c>
       <c r="J25" s="44" t="n">
         <f aca="false">Presupuesto!K421</f>
-        <v>226.75</v>
+        <v>224.05</v>
       </c>
       <c r="K25" s="29" t="n">
         <f aca="false">J25-I25</f>
-        <v>226.75</v>
+        <v>224.05</v>
       </c>
       <c r="L25" s="26" t="s">
         <v>1283</v>
@@ -28565,15 +28565,15 @@
         <v>163</v>
       </c>
       <c r="E28" s="42" t="n">
-        <v>221.12</v>
+        <v>220.41</v>
       </c>
       <c r="F28" s="29" t="n">
         <f aca="false">E28-D28</f>
-        <v>58.12</v>
+        <v>57.41</v>
       </c>
       <c r="G28" s="43" t="n">
         <f aca="false">IF(D28=0,"-",F28/D28)</f>
-        <v>0.356564417177914</v>
+        <v>0.352208588957055</v>
       </c>
       <c r="H28" s="44" t="n">
         <f aca="false">Presupuesto!J437</f>
@@ -28585,11 +28585,11 @@
       </c>
       <c r="J28" s="44" t="n">
         <f aca="false">Presupuesto!K437</f>
-        <v>1017.15</v>
+        <v>1013.89</v>
       </c>
       <c r="K28" s="29" t="n">
         <f aca="false">J28-I28</f>
-        <v>267.35</v>
+        <v>264.09</v>
       </c>
       <c r="L28" s="26" t="s">
         <v>1286</v>
@@ -28612,11 +28612,11 @@
         <v>0</v>
       </c>
       <c r="E29" s="42" t="n">
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="F29" s="29" t="n">
         <f aca="false">E29-D29</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="G29" s="43" t="str">
         <f aca="false">IF(D29=0,"-",F29/D29)</f>
@@ -28632,11 +28632,11 @@
       </c>
       <c r="J29" s="44" t="n">
         <f aca="false">Presupuesto!K457</f>
-        <v>1555.84</v>
+        <v>1540.22</v>
       </c>
       <c r="K29" s="29" t="n">
         <f aca="false">J29-I29</f>
-        <v>1555.84</v>
+        <v>1540.22</v>
       </c>
       <c r="L29" s="26" t="s">
         <v>1287</v>
@@ -28659,15 +28659,15 @@
         <v>99.35</v>
       </c>
       <c r="E30" s="42" t="n">
-        <v>88.43</v>
+        <v>88.49</v>
       </c>
       <c r="F30" s="29" t="n">
         <f aca="false">E30-D30</f>
-        <v>-10.92</v>
+        <v>-10.86</v>
       </c>
       <c r="G30" s="43" t="n">
         <f aca="false">IF(D30=0,"-",F30/D30)</f>
-        <v>-0.109914443885254</v>
+        <v>-0.109310518369401</v>
       </c>
       <c r="H30" s="44" t="n">
         <f aca="false">Presupuesto!J464</f>
@@ -28679,11 +28679,11 @@
       </c>
       <c r="J30" s="44" t="n">
         <f aca="false">Presupuesto!K464</f>
-        <v>2387.61</v>
+        <v>2389.23</v>
       </c>
       <c r="K30" s="29" t="n">
         <f aca="false">J30-I30</f>
-        <v>-294.84</v>
+        <v>-293.22</v>
       </c>
       <c r="L30" s="26" t="s">
         <v>1288</v>
@@ -28847,15 +28847,15 @@
         <v>91.93</v>
       </c>
       <c r="E34" s="42" t="n">
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="F34" s="29" t="n">
         <f aca="false">E34-D34</f>
-        <v>-21.21</v>
+        <v>-21.92</v>
       </c>
       <c r="G34" s="43" t="n">
         <f aca="false">IF(D34=0,"-",F34/D34)</f>
-        <v>-0.230719025345372</v>
+        <v>-0.238442293049059</v>
       </c>
       <c r="H34" s="44" t="n">
         <f aca="false">Presupuesto!J493</f>
@@ -28867,11 +28867,11 @@
       </c>
       <c r="J34" s="44" t="n">
         <f aca="false">Presupuesto!K493</f>
-        <v>3960.32</v>
+        <v>3920.56</v>
       </c>
       <c r="K34" s="29" t="n">
         <f aca="false">J34-I34</f>
-        <v>-1187.76</v>
+        <v>-1227.52</v>
       </c>
       <c r="L34" s="26" t="s">
         <v>1292</v>
@@ -28988,11 +28988,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="42" t="n">
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="F37" s="29" t="n">
         <f aca="false">E37-D37</f>
-        <v>70.72</v>
+        <v>70.01</v>
       </c>
       <c r="G37" s="43" t="str">
         <f aca="false">IF(D37=0,"-",F37/D37)</f>
@@ -29008,11 +29008,11 @@
       </c>
       <c r="J37" s="44" t="n">
         <f aca="false">Presupuesto!K513</f>
-        <v>1060.8</v>
+        <v>1050.15</v>
       </c>
       <c r="K37" s="29" t="n">
         <f aca="false">J37-I37</f>
-        <v>1060.8</v>
+        <v>1050.15</v>
       </c>
       <c r="L37" s="26" t="s">
         <v>1293</v>
@@ -29035,15 +29035,15 @@
         <v>196.3</v>
       </c>
       <c r="E38" s="42" t="n">
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="F38" s="29" t="n">
         <f aca="false">E38-D38</f>
-        <v>112.19</v>
+        <v>125.99</v>
       </c>
       <c r="G38" s="43" t="n">
         <f aca="false">IF(D38=0,"-",F38/D38)</f>
-        <v>0.571523178807947</v>
+        <v>0.641823739174733</v>
       </c>
       <c r="H38" s="44" t="n">
         <f aca="false">Presupuesto!J522</f>
@@ -29055,11 +29055,11 @@
       </c>
       <c r="J38" s="44" t="n">
         <f aca="false">Presupuesto!K522</f>
-        <v>9118.96</v>
+        <v>9526.89</v>
       </c>
       <c r="K38" s="29" t="n">
         <f aca="false">J38-I38</f>
-        <v>3316.33</v>
+        <v>3724.26</v>
       </c>
       <c r="L38" s="26" t="s">
         <v>1294</v>
@@ -29082,15 +29082,15 @@
         <v>701.6</v>
       </c>
       <c r="E39" s="42" t="n">
-        <v>947.29</v>
+        <v>950.13</v>
       </c>
       <c r="F39" s="29" t="n">
         <f aca="false">E39-D39</f>
-        <v>245.69</v>
+        <v>248.53</v>
       </c>
       <c r="G39" s="43" t="n">
         <f aca="false">IF(D39=0,"-",F39/D39)</f>
-        <v>0.350185290763968</v>
+        <v>0.354233181299886</v>
       </c>
       <c r="H39" s="44" t="n">
         <f aca="false">Presupuesto!J532</f>
@@ -29102,11 +29102,11 @@
       </c>
       <c r="J39" s="44" t="n">
         <f aca="false">Presupuesto!K532</f>
-        <v>13262.06</v>
+        <v>13301.82</v>
       </c>
       <c r="K39" s="29" t="n">
         <f aca="false">J39-I39</f>
-        <v>3439.66</v>
+        <v>3479.42</v>
       </c>
       <c r="L39" s="26" t="s">
         <v>1295</v>
@@ -29129,15 +29129,15 @@
         <v>67.81</v>
       </c>
       <c r="E40" s="42" t="n">
-        <v>88.58</v>
+        <v>88.02</v>
       </c>
       <c r="F40" s="29" t="n">
         <f aca="false">E40-D40</f>
-        <v>20.77</v>
+        <v>20.21</v>
       </c>
       <c r="G40" s="43" t="n">
         <f aca="false">IF(D40=0,"-",F40/D40)</f>
-        <v>0.306297006341248</v>
+        <v>0.29803863736912</v>
       </c>
       <c r="H40" s="44" t="n">
         <f aca="false">Presupuesto!J540</f>
@@ -29149,11 +29149,11 @@
       </c>
       <c r="J40" s="44" t="n">
         <f aca="false">Presupuesto!K540</f>
-        <v>5669.12</v>
+        <v>5633.28</v>
       </c>
       <c r="K40" s="29" t="n">
         <f aca="false">J40-I40</f>
-        <v>1329.28</v>
+        <v>1293.44</v>
       </c>
       <c r="L40" s="26" t="s">
         <v>1296</v>
@@ -29928,15 +29928,15 @@
         <v>818.95</v>
       </c>
       <c r="E57" s="42" t="n">
-        <v>1035.72</v>
+        <v>1038.62</v>
       </c>
       <c r="F57" s="29" t="n">
         <f aca="false">E57-D57</f>
-        <v>216.77</v>
+        <v>219.67</v>
       </c>
       <c r="G57" s="43" t="n">
         <f aca="false">IF(D57=0,"-",F57/D57)</f>
-        <v>0.264692594175469</v>
+        <v>0.268233713901947</v>
       </c>
       <c r="H57" s="44" t="n">
         <f aca="false">Presupuesto!J671</f>
@@ -29948,11 +29948,11 @@
       </c>
       <c r="J57" s="44" t="n">
         <f aca="false">Presupuesto!K671</f>
-        <v>6597.54</v>
+        <v>6616.01</v>
       </c>
       <c r="K57" s="29" t="n">
         <f aca="false">J57-I57</f>
-        <v>1380.83</v>
+        <v>1399.3</v>
       </c>
       <c r="L57" s="26" t="s">
         <v>1311</v>
@@ -29975,15 +29975,15 @@
         <v>196.3</v>
       </c>
       <c r="E58" s="42" t="n">
-        <v>308.49</v>
+        <v>322.29</v>
       </c>
       <c r="F58" s="29" t="n">
         <f aca="false">E58-D58</f>
-        <v>112.19</v>
+        <v>125.99</v>
       </c>
       <c r="G58" s="43" t="n">
         <f aca="false">IF(D58=0,"-",F58/D58)</f>
-        <v>0.571523178807947</v>
+        <v>0.641823739174733</v>
       </c>
       <c r="H58" s="44" t="n">
         <f aca="false">Presupuesto!J675</f>
@@ -29995,11 +29995,11 @@
       </c>
       <c r="J58" s="44" t="n">
         <f aca="false">Presupuesto!K675</f>
-        <v>2329.1</v>
+        <v>2433.29</v>
       </c>
       <c r="K58" s="29" t="n">
         <f aca="false">J58-I58</f>
-        <v>847.03</v>
+        <v>951.22</v>
       </c>
       <c r="L58" s="26" t="s">
         <v>1312</v>
@@ -30015,11 +30015,11 @@
       </c>
       <c r="J60" s="45" t="n">
         <f aca="false">SUM(J6:J58)</f>
-        <v>217059.78</v>
+        <v>217751.11</v>
       </c>
       <c r="K60" s="45" t="n">
         <f aca="false">SUM(K6:K58)</f>
-        <v>9599.93</v>
+        <v>10291.26</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30036,7 +30036,7 @@
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">Resumen!C48</f>
-        <v>361925.63</v>
+        <v>362644.27</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30045,7 +30045,7 @@
       </c>
       <c r="J64" s="45" t="n">
         <f aca="false">J63-J62</f>
-        <v>2722.60999999993</v>
+        <v>3441.24999999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Visor: lodosa (2026-10-21 23:18)
</commit_message>
<xml_diff>
--- a/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
+++ b/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
@@ -3784,7 +3784,7 @@
     <t xml:space="preserve">Opción 3 de cubiertas · IFC final (21-oct)</t>
   </si>
   <si>
-    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261021-2001.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (322,29 m², con 13,43 m² de cantos de losas y faldones que quedaban vistos; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta hasta la pared (24,39 m en total). La unidad exterior de la aerotermia vuelve a la cubierta plana. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement).</t>
+    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261021-2238.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (310,64 m²: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos, sin contar dos veces lo que se solapaba; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta hasta la pared (24,39 m en total). La unidad exterior de la aerotermia vuelve a la cubierta plana. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement). IFC 22:38 (Enrique 21-oct, «el mortero es continuo»): los paños de revoco del mismo plano forman uno solo (con los cantos de losas y faldones) y la junta de poliestireno de las medianeras solo va contra la casa vecina: donde la medianera asoma por encima del vecino y lleva revoco, no hay junta.</t>
   </si>
   <si>
     <t xml:space="preserve">MEDICIONES DEL MODELO BIM FRENTE A LA PROPUESTA DE OCTUBRE</t>
@@ -3853,7 +3853,7 @@
     <t xml:space="preserve">Medianeras M2–M5/M10–M12 e interiores de carga M13 · Opción 2 de cubiertas (16-oct): +8,09 m² de medianera M2 que sube hasta el faldón sobre la escalera y +2,54 m² de M13 (muro de la escalera hasta el alféizar del ventanal y dintel encima) · Opción 3 de cubiertas, IFC final (21-oct): +7,09 m² de la medianera M2 que sube hasta el faldón a la medianera oeste, +2,62 m² de muro de carga M13/M13b y −0,37 m² de recortes · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): −1,49 m²: el muro de 45 cm del baño de segunda y de la cocina pasa a ser de carga de 20 cm + trasdosado (M13t, Enrique 21-oct), medianeras y muros de carga remedidos</t>
   </si>
   <si>
-    <t xml:space="preserve">Capa de junta de los muros de medianera · Opción 2 de cubiertas (16-oct): +8,09 m² de la medianera M2 que sube hasta el faldón sobre la escalera · Opción 3 de cubiertas, IFC final (21-oct): +6,72 m² de junta de las medianeras (la M2 que sube). Se mide con la geometría. En el IFC 1843 la junta sale en todas las medianeras como capa del muro · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): −0,23 m² de medianera de segunda (IFC 20:01)</t>
+    <t xml:space="preserve">Capa de junta de los muros de medianera · Opción 2 de cubiertas (16-oct): +8,09 m² de la medianera M2 que sube hasta el faldón sobre la escalera · Opción 3 de cubiertas, IFC final (21-oct): +6,72 m² de junta de las medianeras (la M2 que sube). Se mide con la geometría. En el IFC 1843 la junta sale en todas las medianeras como capa del muro · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): −0,23 m² de medianera de segunda (IFC 20:01) · IFC 22:38 (21-oct, mortero continuo): junta solo donde la fábrica va contra la casa vecina: −38,68 m² en los tramos de medianera que asoman por encima del vecino y llevan revoco (oeste de planta baja y primera, segunda sobre V2, V4 y V6)</t>
   </si>
   <si>
     <t xml:space="preserve">Muros M4/M5/M6 (trasdosado de 7 cm con cámara) · Opción 3 de cubiertas, IFC final (21-oct): −2,09 m² (M6 de primera y segunda) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +3,60 m² del trasdosado del muro de carga del baño de segunda y de la cocina (M13t)</t>
@@ -3910,7 +3910,7 @@
     <t xml:space="preserve">Patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 29,31 m²</t>
   </si>
   <si>
-    <t xml:space="preserve">Caras revocadas de muros exteriores y frentes de forjado · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro y +0,68 m² de frente de forjado · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): revoco continuo del IFC (piel vista de la casa, 34 paños de arriba abajo, regla de Enrique del 19 y 21-oct): caras 289,80 m² con los huecos descontados + mochetas y dinteles 18,68 m²; sin medianeras, bajo aleros ni zócalo. Sustituye a la medición por caras de muro (261,81) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): revoco continuo del IFC 20:01: paños de fachada 308,86 m² + cantos de losas y faldones que quedaban vistos 13,43 m² (patinillo, bordes de la cubierta plana, terraza de segunda, faldones sobre la terraza; Enrique 21-oct: el mortero es continuo)</t>
+    <t xml:space="preserve">Caras revocadas de muros exteriores y frentes de forjado · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro y +0,68 m² de frente de forjado · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): revoco continuo del IFC (piel vista de la casa, 34 paños de arriba abajo, regla de Enrique del 19 y 21-oct): caras 289,80 m² con los huecos descontados + mochetas y dinteles 18,68 m²; sin medianeras, bajo aleros ni zócalo. Sustituye a la medición por caras de muro (261,81) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): revoco continuo del IFC 20:01: paños de fachada 308,86 m² + cantos de losas y faldones que quedaban vistos 13,43 m² (patinillo, bordes de la cubierta plana, terraza de segunda, faldones sobre la terraza; Enrique 21-oct: el mortero es continuo) · IFC 22:38 (21-oct, mortero continuo): revoco continuo del IFC 22:38: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos (cara 291,79 m² + mochetas y dinteles 18,85 m²); −11,65 m² respecto al IFC 20:01, que contaba dos veces los cantos tapados por el paño</t>
   </si>
   <si>
     <t xml:space="preserve">Paredes 726.4 m² (incluye 27.6 m² de baños y aseos por encima de 2,28 m) y techos sin falso techo 214.4 m² · Opción 2 de cubiertas (16-oct): paredes: +8,09 medianera M2, +5,08 muro M13 (dos caras), −4,72 tabique T2 (dos caras), −1,50 quiebro; techos: −8,52 m² que pasan a falso techo · Opción 3 de cubiertas, IFC final (21-oct): paredes −0,80 m² (cambios de muros de segunda) y techos +8,89 m²: bajo el faldón de la escalera ya no hay falso techo (+8,52) y el faldón a la medianera oeste tiene más superficie en pendiente que la cubierta plana a la que sustituye (+0,37) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +2,84 m² de yeso en paredes (muros de segunda remedidos y trasdosado M13t)</t>
@@ -3964,7 +3964,7 @@
     <t xml:space="preserve">Yeso de paredes y techos más falsos techos · Opción 2 de cubiertas (16-oct): yeso 939,20 + falsos techos 96,96 · Opción 3 de cubiertas, IFC final (21-oct): yeso 947,29 + falsos techos 88,43 · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): yeso 950,13 + falsos techos 88,49</t>
   </si>
   <si>
-    <t xml:space="preserve">Igual que el revoco · Opción 2 de cubiertas (16-oct): igual que el revoco · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): igual que el revoco · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): igual que el revoco</t>
+    <t xml:space="preserve">Igual que el revoco · Opción 2 de cubiertas (16-oct): igual que el revoco · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): igual que el revoco · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): igual que el revoco · IFC 22:38 (21-oct, mortero continuo): igual que el revoco</t>
   </si>
   <si>
     <t xml:space="preserve">Total de las partidas medidas con el BIM</t>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C7/$C$50)</f>
-        <v>0.00248239800897721</v>
+        <v>0.00248639966511337</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C8/$C$50)</f>
-        <v>0.02420046379591</v>
+        <v>0.0242394752413336</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C9/$C$50)</f>
-        <v>0.0251143571124336</v>
+        <v>0.0251548417651288</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C10/$C$50)</f>
-        <v>0.0037762034337148</v>
+        <v>0.00378229072011581</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C14/$C$50)</f>
-        <v>0.00398688954253379</v>
+        <v>0.00399331645753468</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C16/$C$50)</f>
-        <v>0.0130889200852484</v>
+        <v>0.0131100195854839</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C17/$C$50)</f>
-        <v>0.0168807752311264</v>
+        <v>0.0169079872485155</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C18/$C$50)</f>
-        <v>0.187202837204875</v>
+        <v>0.187504610481964</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4856,11 +4856,11 @@
       </c>
       <c r="C21" s="8" t="n">
         <f aca="false">Presupuesto!K365</f>
-        <v>56216.97</v>
+        <v>56031.31</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C21/$C$50)</f>
-        <v>0.146404631135891</v>
+        <v>0.146156347482022</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C22/$C$50)</f>
-        <v>0.0374673081698422</v>
+        <v>0.0375277059316439</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C23/$C$50)</f>
-        <v>0.0196142256614899</v>
+        <v>0.0196458440346076</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C24/$C$50)</f>
-        <v>0.00957184233543338</v>
+        <v>0.00958727226305879</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C25/$C$50)</f>
-        <v>0.0566813343957052</v>
+        <v>0.05677270540421</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4936,11 +4936,11 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">Presupuesto!K545</f>
-        <v>28920.71</v>
+        <v>28576.34</v>
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C26/$C$50)</f>
-        <v>0.0753175754534276</v>
+        <v>0.0745407073081891</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C27/$C$50)</f>
-        <v>0.0275290959729916</v>
+        <v>0.0275734732144432</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C28/$C$50)</f>
-        <v>0.13690432832344</v>
+        <v>0.137125019785293</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C29/$C$50)</f>
-        <v>0.0535860195052627</v>
+        <v>0.0536724008280765</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">Presupuesto!K676</f>
-        <v>9049.3</v>
+        <v>8961.34</v>
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C30/$C$50)</f>
-        <v>0.0235668949880796</v>
+        <v>0.0233754435322776</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C31/$C$50)</f>
-        <v>0.114825726258325</v>
+        <v>0.115010826741974</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C38/$C$50)</f>
-        <v>0.00397022216186084</v>
+        <v>0.003976622208839</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C41/$C$50)</f>
-        <v>0.00716186930403659</v>
+        <v>0.00717341432548088</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="D42" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C42/$C$50)</f>
-        <v>0.0106660819193947</v>
+        <v>0.010683275774694</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="C48" s="10" t="n">
         <f aca="false">C14+C15+C16+C17+C18+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C38+C41+C42</f>
-        <v>362644.27</v>
+        <v>362026.28</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="C50" s="14" t="n">
         <f aca="false">C11+C48</f>
-        <v>383983.55</v>
+        <v>383365.56</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="C52" s="15" t="n">
         <f aca="false">ROUND(C50*D52,2)</f>
-        <v>19199.18</v>
+        <v>19168.28</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>0.05</v>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="C53" s="15" t="n">
         <f aca="false">ROUND(C50*D53,2)</f>
-        <v>19199.18</v>
+        <v>19168.28</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>0.05</v>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">C50+C52+C53</f>
-        <v>422381.91</v>
+        <v>421702.12</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="C56" s="15" t="n">
         <f aca="false">ROUND(C48*(1+$D$52+$D$53)*D56,2)</f>
-        <v>39890.87</v>
+        <v>39822.89</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>0.1</v>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C57" s="14" t="n">
         <f aca="false">C54+C55+C56</f>
-        <v>467202.15</v>
+        <v>466454.38</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="C61" s="15" t="n">
         <f aca="false">C50/C60</f>
-        <v>1093.4095050971</v>
+        <v>1091.6497522638</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10337,12 +10337,12 @@
       </c>
       <c r="E317" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E17</f>
-        <v>366.74</v>
+        <v>328.06</v>
       </c>
       <c r="G317" s="28"/>
       <c r="H317" s="29" t="n">
         <f aca="false">IF(COUNT(D317:G317)=0,0,D317*IF(E317="",1,E317)*IF(F317="",1,F317)*IF(G317="",1,G317))</f>
-        <v>366.74</v>
+        <v>328.06</v>
       </c>
       <c r="M317" s="23"/>
       <c r="N317" s="23"/>
@@ -10378,14 +10378,14 @@
       <c r="H320" s="30"/>
       <c r="I320" s="31" t="n">
         <f aca="false">ROUND(SUM(H317:H319),2)</f>
-        <v>366.74</v>
+        <v>328.06</v>
       </c>
       <c r="J320" s="32" t="n">
         <v>4.8</v>
       </c>
       <c r="K320" s="31" t="n">
         <f aca="false">ROUND(I320*J320,2)</f>
-        <v>1760.35</v>
+        <v>1574.69</v>
       </c>
       <c r="L320" s="33" t="s">
         <v>238</v>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="K365" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$364,$M$5:$M$364,"P",$N$5:$N$364,"06")</f>
-        <v>56216.97</v>
+        <v>56031.31</v>
       </c>
       <c r="M365" s="23"/>
       <c r="N365" s="23"/>
@@ -13515,11 +13515,11 @@
       </c>
       <c r="E519" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E38</f>
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="H519" s="29" t="n">
         <f aca="false">IF(COUNT(D519:G519)=0,0,D519*IF(E519="",1,E519)*IF(F519="",1,F519)*IF(G519="",1,G519))</f>
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="M519" s="23"/>
       <c r="N519" s="23"/>
@@ -13553,14 +13553,14 @@
       <c r="H522" s="30"/>
       <c r="I522" s="31" t="n">
         <f aca="false">ROUND(SUM(H519:H521),2)</f>
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="J522" s="32" t="n">
         <v>29.56</v>
       </c>
       <c r="K522" s="31" t="n">
         <f aca="false">ROUND(I522*J522,2)</f>
-        <v>9526.89</v>
+        <v>9182.52</v>
       </c>
       <c r="L522" s="33" t="s">
         <v>212</v>
@@ -13898,7 +13898,7 @@
       </c>
       <c r="K545" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$544,$M$5:$M$544,"P",$N$5:$N$544,"11")</f>
-        <v>28920.71</v>
+        <v>28576.34</v>
       </c>
       <c r="M545" s="23"/>
       <c r="N545" s="23"/>
@@ -15918,11 +15918,11 @@
       </c>
       <c r="E674" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E58</f>
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="H674" s="29" t="n">
         <f aca="false">IF(COUNT(D674:G674)=0,0,D674*IF(E674="",1,E674)*IF(F674="",1,F674)*IF(G674="",1,G674))</f>
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="M674" s="23"/>
       <c r="N674" s="23"/>
@@ -15932,14 +15932,14 @@
       <c r="H675" s="30"/>
       <c r="I675" s="31" t="n">
         <f aca="false">ROUND(SUM(H674:H674),2)</f>
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="J675" s="32" t="n">
         <v>7.55</v>
       </c>
       <c r="K675" s="31" t="n">
         <f aca="false">ROUND(I675*J675,2)</f>
-        <v>2433.29</v>
+        <v>2345.33</v>
       </c>
       <c r="L675" s="33" t="s">
         <v>212</v>
@@ -15958,7 +15958,7 @@
       </c>
       <c r="K676" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$675,$M$5:$M$675,"P",$N$5:$N$675,"15")</f>
-        <v>9049.3</v>
+        <v>8961.34</v>
       </c>
       <c r="M676" s="23"/>
       <c r="N676" s="23"/>
@@ -28049,15 +28049,15 @@
         <v>350.03</v>
       </c>
       <c r="E17" s="42" t="n">
-        <v>366.74</v>
+        <v>328.06</v>
       </c>
       <c r="F17" s="29" t="n">
         <f aca="false">E17-D17</f>
-        <v>16.71</v>
+        <v>-21.97</v>
       </c>
       <c r="G17" s="43" t="n">
         <f aca="false">IF(D17=0,"-",F17/D17)</f>
-        <v>0.0477387652486931</v>
+        <v>-0.0627660486244036</v>
       </c>
       <c r="H17" s="44" t="n">
         <f aca="false">Presupuesto!J320</f>
@@ -28069,11 +28069,11 @@
       </c>
       <c r="J17" s="44" t="n">
         <f aca="false">Presupuesto!K320</f>
-        <v>1760.35</v>
+        <v>1574.69</v>
       </c>
       <c r="K17" s="29" t="n">
         <f aca="false">J17-I17</f>
-        <v>80.2099999999998</v>
+        <v>-105.45</v>
       </c>
       <c r="L17" s="26" t="s">
         <v>1275</v>
@@ -29035,15 +29035,15 @@
         <v>196.3</v>
       </c>
       <c r="E38" s="42" t="n">
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="F38" s="29" t="n">
         <f aca="false">E38-D38</f>
-        <v>125.99</v>
+        <v>114.34</v>
       </c>
       <c r="G38" s="43" t="n">
         <f aca="false">IF(D38=0,"-",F38/D38)</f>
-        <v>0.641823739174733</v>
+        <v>0.582475802343352</v>
       </c>
       <c r="H38" s="44" t="n">
         <f aca="false">Presupuesto!J522</f>
@@ -29055,11 +29055,11 @@
       </c>
       <c r="J38" s="44" t="n">
         <f aca="false">Presupuesto!K522</f>
-        <v>9526.89</v>
+        <v>9182.52</v>
       </c>
       <c r="K38" s="29" t="n">
         <f aca="false">J38-I38</f>
-        <v>3724.26</v>
+        <v>3379.89</v>
       </c>
       <c r="L38" s="26" t="s">
         <v>1294</v>
@@ -29975,15 +29975,15 @@
         <v>196.3</v>
       </c>
       <c r="E58" s="42" t="n">
-        <v>322.29</v>
+        <v>310.64</v>
       </c>
       <c r="F58" s="29" t="n">
         <f aca="false">E58-D58</f>
-        <v>125.99</v>
+        <v>114.34</v>
       </c>
       <c r="G58" s="43" t="n">
         <f aca="false">IF(D58=0,"-",F58/D58)</f>
-        <v>0.641823739174733</v>
+        <v>0.582475802343352</v>
       </c>
       <c r="H58" s="44" t="n">
         <f aca="false">Presupuesto!J675</f>
@@ -29995,11 +29995,11 @@
       </c>
       <c r="J58" s="44" t="n">
         <f aca="false">Presupuesto!K675</f>
-        <v>2433.29</v>
+        <v>2345.33</v>
       </c>
       <c r="K58" s="29" t="n">
         <f aca="false">J58-I58</f>
-        <v>951.22</v>
+        <v>863.26</v>
       </c>
       <c r="L58" s="26" t="s">
         <v>1312</v>
@@ -30015,11 +30015,11 @@
       </c>
       <c r="J60" s="45" t="n">
         <f aca="false">SUM(J6:J58)</f>
-        <v>217751.11</v>
+        <v>217133.12</v>
       </c>
       <c r="K60" s="45" t="n">
         <f aca="false">SUM(K6:K58)</f>
-        <v>10291.26</v>
+        <v>9673.27000000001</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30036,7 +30036,7 @@
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">Resumen!C48</f>
-        <v>362644.27</v>
+        <v>362026.28</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30045,7 +30045,7 @@
       </c>
       <c r="J64" s="45" t="n">
         <f aca="false">J63-J62</f>
-        <v>3441.24999999994</v>
+        <v>2823.26000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Visor: lodosa (2026-10-22 01:31)
</commit_message>
<xml_diff>
--- a/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
+++ b/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
@@ -2221,7 +2221,7 @@
     <t xml:space="preserve">BOMBA DE CALOR AIRE-AGUA 8 KW CON DEPÓSITO DE ACS 230 L</t>
   </si>
   <si>
-    <t xml:space="preserve">Bomba de calor aire-agua de baja temperatura tipo Daikin Altherma 3 de 8 kW (SCOP 4,61 a 35 °C, A+++), unidad exterior en la cubierta plana, sobre bancada antivibratoria y unidad interior con depósito de ACS de 230 L y resistencia de apoyo integrada en el almacenaje de planta baja, con puesta en marcha.</t>
+    <t xml:space="preserve">Bomba de calor aire-agua de baja temperatura tipo Daikin Altherma 3 de 8 kW (SCOP 4,61 a 35 °C, A+++), unidad exterior en el hueco del muro grueso de la cubierta, junto al V12, sobre bancada antivibratoria, ventilada y registrable desde la terraza, sobre bancada antivibratoria y unidad interior con depósito de ACS de 230 L y resistencia de apoyo integrada en el almacenaje de planta baja, con puesta en marcha.</t>
   </si>
   <si>
     <t xml:space="preserve">Almacenaje de planta baja / cubierta</t>
@@ -3784,7 +3784,7 @@
     <t xml:space="preserve">Opción 3 de cubiertas · IFC final (21-oct)</t>
   </si>
   <si>
-    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261021-2238.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (310,64 m²: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos, sin contar dos veces lo que se solapaba; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta hasta la pared (24,39 m en total). La unidad exterior de la aerotermia vuelve a la cubierta plana. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement). IFC 22:38 (Enrique 21-oct, «el mortero es continuo»): los paños de revoco del mismo plano forman uno solo (con los cantos de losas y faldones) y la junta de poliestireno de las medianeras solo va contra la casa vecina: donde la medianera asoma por encima del vecino y lleva revoco, no hay junta.</t>
+    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261022-0051.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (310,64 m²: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos, sin contar dos veces lo que se solapaba; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta, por detrás de la arista del faldón y no al borde del muro (Enrique 22-oct; 24,08 m en total). La unidad exterior de la aerotermia va en el hueco del muro grueso de la cubierta, junto al V12, ventilada y registrable desde la terraza (Enrique 22-oct); la puerta perforada contigua al V12 está en propuesta (hoja LO-G3b) y todavía no tiene partida. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement). IFC 22:38 (Enrique 21-oct, «el mortero es continuo»): los paños de revoco del mismo plano forman uno solo (con los cantos de losas y faldones) y la junta de poliestireno de las medianeras solo va contra la casa vecina: donde la medianera asoma por encima del vecino y lleva revoco, no hay junta. IFC 00:51 (22-oct): la barandilla del patio en cubierta pasa por detrás de la arista del faldón (−0,31 m) y la unidad exterior de la aerotermia, al muro grueso junto al V12. El modelo lleva además las instalaciones en 3D (líneas sin medición ni IFC), que no cambian el presupuesto.</t>
   </si>
   <si>
     <t xml:space="preserve">MEDICIONES DEL MODELO BIM FRENTE A LA PROPUESTA DE OCTUBRE</t>
@@ -3955,7 +3955,7 @@
     <t xml:space="preserve">V11 (1,80 m en el BIM)</t>
   </si>
   <si>
-    <t xml:space="preserve">Longitud del eje de la barandilla en el BIM: cubierta → patio 9.99 m (h 1.10); patio pequeño (hueco del ascensor) en cubierta 4.91 m (h 1.10); terraza de segunda → patio 4.04 m (h 1.10). Sustituye a la estimación de la propuesta (terraza en cubierta 15 + terraza de segunda 8 + patio pequeño 3 m) · Opción 2 de cubiertas (16-oct): cubierta → patio 9,99 m + terraza de segunda → patio 4,04 m + barandilla nueva de la zona pisable de la cubierta (escalera y terraza) 13,05 m; ya no lleva la del patio pequeño en cubierta (4,91 m) · Opción 3 de cubiertas, IFC final (21-oct): IFC: terraza de segunda → patio 4,04 + zona pisable de la cubierta (escalera y terraza) 13,05 + cubierta → patio 7,30 m (borde norte del patio recto hasta la pared, sin vuelta por el borde oeste, que ahora es faldón)</t>
+    <t xml:space="preserve">Longitud del eje de la barandilla en el BIM: cubierta → patio 9.99 m (h 1.10); patio pequeño (hueco del ascensor) en cubierta 4.91 m (h 1.10); terraza de segunda → patio 4.04 m (h 1.10). Sustituye a la estimación de la propuesta (terraza en cubierta 15 + terraza de segunda 8 + patio pequeño 3 m) · Opción 2 de cubiertas (16-oct): cubierta → patio 9,99 m + terraza de segunda → patio 4,04 m + barandilla nueva de la zona pisable de la cubierta (escalera y terraza) 13,05 m; ya no lleva la del patio pequeño en cubierta (4,91 m) · Opción 3 de cubiertas, IFC final (21-oct): IFC: terraza de segunda → patio 4,04 + zona pisable de la cubierta (escalera y terraza) 13,05 + cubierta → patio 7,30 m (borde norte del patio recto hasta la pared, sin vuelta por el borde oeste, que ahora es faldón) · IFC 00:51 (22-oct): IFC 00:51: terraza de segunda → patio 4,04 + zona pisable de la cubierta 12,80 + cubierta → patio 7,24 m: la barandilla del borde norte del patio pasa recta por detrás de la arista del faldón, no al borde del muro (Enrique 22-oct)</t>
   </si>
   <si>
     <t xml:space="preserve">Mini-balcones de V1, V2 y V3</t>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C7/$C$50)</f>
-        <v>0.00248639966511337</v>
+        <v>0.00248683201316696</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C8/$C$50)</f>
-        <v>0.0242394752413336</v>
+        <v>0.0242436901268517</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C9/$C$50)</f>
-        <v>0.0251548417651288</v>
+        <v>0.0251592158193197</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C10/$C$50)</f>
-        <v>0.00378229072011581</v>
+        <v>0.00378294840441889</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C14/$C$50)</f>
-        <v>0.00399331645753468</v>
+        <v>0.00399401083608612</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C16/$C$50)</f>
-        <v>0.0131100195854839</v>
+        <v>0.0131122992236007</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C17/$C$50)</f>
-        <v>0.0169079872485155</v>
+        <v>0.0169109272969234</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C18/$C$50)</f>
-        <v>0.187504610481964</v>
+        <v>0.187537214754928</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C21/$C$50)</f>
-        <v>0.146156347482022</v>
+        <v>0.146181761904828</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C22/$C$50)</f>
-        <v>0.0375277059316439</v>
+        <v>0.0375342314435488</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C23/$C$50)</f>
-        <v>0.0196458440346076</v>
+        <v>0.0196492601557359</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C24/$C$50)</f>
-        <v>0.00958727226305879</v>
+        <v>0.00958893934762298</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C25/$C$50)</f>
-        <v>0.05677270540421</v>
+        <v>0.0567825773363144</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C26/$C$50)</f>
-        <v>0.0745407073081891</v>
+        <v>0.0745536688325046</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C27/$C$50)</f>
-        <v>0.0275734732144432</v>
+        <v>0.0275782678327992</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C28/$C$50)</f>
-        <v>0.137125019785293</v>
+        <v>0.137148863794056</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4984,11 +4984,11 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">Presupuesto!K664</f>
-        <v>20576.15</v>
+        <v>20509.5</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C29/$C$50)</f>
-        <v>0.0536724008280765</v>
+        <v>0.0535078484830546</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C30/$C$50)</f>
-        <v>0.0233754435322776</v>
+        <v>0.0233795081754863</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C31/$C$50)</f>
-        <v>0.115010826741974</v>
+        <v>0.115030825420297</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C38/$C$50)</f>
-        <v>0.003976622208839</v>
+        <v>0.003977313684508</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C41/$C$50)</f>
-        <v>0.00717341432548088</v>
+        <v>0.00717466167592285</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="D42" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C42/$C$50)</f>
-        <v>0.010683275774694</v>
+        <v>0.0106851334380262</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="C48" s="10" t="n">
         <f aca="false">C14+C15+C16+C17+C18+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C38+C41+C42</f>
-        <v>362026.28</v>
+        <v>361959.63</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="C50" s="14" t="n">
         <f aca="false">C11+C48</f>
-        <v>383365.56</v>
+        <v>383298.91</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="C52" s="15" t="n">
         <f aca="false">ROUND(C50*D52,2)</f>
-        <v>19168.28</v>
+        <v>19164.95</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>0.05</v>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="C53" s="15" t="n">
         <f aca="false">ROUND(C50*D53,2)</f>
-        <v>19168.28</v>
+        <v>19164.95</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>0.05</v>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">C50+C52+C53</f>
-        <v>421702.12</v>
+        <v>421628.81</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="C56" s="15" t="n">
         <f aca="false">ROUND(C48*(1+$D$52+$D$53)*D56,2)</f>
-        <v>39822.89</v>
+        <v>39815.56</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>0.1</v>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C57" s="14" t="n">
         <f aca="false">C54+C55+C56</f>
-        <v>466454.38</v>
+        <v>466373.74</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="C61" s="15" t="n">
         <f aca="false">C50/C60</f>
-        <v>1091.6497522638</v>
+        <v>1091.45996355146</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15519,11 +15519,11 @@
       </c>
       <c r="E648" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E55</f>
-        <v>24.39</v>
+        <v>24.08</v>
       </c>
       <c r="H648" s="29" t="n">
         <f aca="false">IF(COUNT(D648:G648)=0,0,D648*IF(E648="",1,E648)*IF(F648="",1,F648)*IF(G648="",1,G648))</f>
-        <v>24.39</v>
+        <v>24.08</v>
       </c>
       <c r="M648" s="23"/>
       <c r="N648" s="23"/>
@@ -15557,14 +15557,14 @@
       <c r="H651" s="30"/>
       <c r="I651" s="31" t="n">
         <f aca="false">ROUND(SUM(H648:H650),2)</f>
-        <v>24.39</v>
+        <v>24.08</v>
       </c>
       <c r="J651" s="32" t="n">
         <v>215</v>
       </c>
       <c r="K651" s="31" t="n">
         <f aca="false">ROUND(I651*J651,2)</f>
-        <v>5243.85</v>
+        <v>5177.2</v>
       </c>
       <c r="L651" s="33" t="s">
         <v>238</v>
@@ -15774,7 +15774,7 @@
       </c>
       <c r="K664" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$663,$M$5:$M$663,"P",$N$5:$N$663,"14")</f>
-        <v>20576.15</v>
+        <v>20509.5</v>
       </c>
       <c r="M664" s="23"/>
       <c r="N664" s="23"/>
@@ -29834,15 +29834,15 @@
         <v>26</v>
       </c>
       <c r="E55" s="42" t="n">
-        <v>24.39</v>
+        <v>24.08</v>
       </c>
       <c r="F55" s="29" t="n">
         <f aca="false">E55-D55</f>
-        <v>-1.61</v>
+        <v>-1.92</v>
       </c>
       <c r="G55" s="43" t="n">
         <f aca="false">IF(D55=0,"-",F55/D55)</f>
-        <v>-0.0619230769230769</v>
+        <v>-0.0738461538461539</v>
       </c>
       <c r="H55" s="44" t="n">
         <f aca="false">Presupuesto!J651</f>
@@ -29854,11 +29854,11 @@
       </c>
       <c r="J55" s="44" t="n">
         <f aca="false">Presupuesto!K651</f>
-        <v>5243.85</v>
+        <v>5177.2</v>
       </c>
       <c r="K55" s="29" t="n">
         <f aca="false">J55-I55</f>
-        <v>-346.15</v>
+        <v>-412.8</v>
       </c>
       <c r="L55" s="26" t="s">
         <v>1309</v>
@@ -30015,11 +30015,11 @@
       </c>
       <c r="J60" s="45" t="n">
         <f aca="false">SUM(J6:J58)</f>
-        <v>217133.12</v>
+        <v>217066.47</v>
       </c>
       <c r="K60" s="45" t="n">
         <f aca="false">SUM(K6:K58)</f>
-        <v>9673.27000000001</v>
+        <v>9606.62000000001</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30036,7 +30036,7 @@
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">Resumen!C48</f>
-        <v>362026.28</v>
+        <v>361959.63</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30045,7 +30045,7 @@
       </c>
       <c r="J64" s="45" t="n">
         <f aca="false">J63-J62</f>
-        <v>2823.26000000001</v>
+        <v>2756.60999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Visor: lodosa (2026-10-22 09:49)
</commit_message>
<xml_diff>
--- a/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
+++ b/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
@@ -2428,7 +2428,7 @@
     <t xml:space="preserve">Rejilla de extracción circular vista de Ø125 mm de aluminio anodizado (tipo Mayfe o la marca que fije la dirección facultativa), enrasada en techo o falso techo, con su marco de montaje y conexión al conducto Ø125.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bocas de extracción de los planos LO-H5 y LO-H6 (11, contadas en el modelo 3D el 22-oct; la campana va aparte)</t>
+    <t xml:space="preserve">Bocas de extracción de los planos LO-H5 y LO-H6 (10, contadas en el modelo 3D el 22-oct; la campana va aparte y la salida de aire de la cámara Cupolex no es boca)</t>
   </si>
   <si>
     <t xml:space="preserve">Precio de referencia de mercado (rejilla Ø125 de aluminio anodizado, montada); contrastar con el fabricante</t>
@@ -2740,7 +2740,7 @@
     <t xml:space="preserve">Punto de ventilacion, empotrado con cable de cobre 07z1-k de 2,5 mm2, 4 mm2 o 6 mm2, segun corresponda al equipo, cero halógenos marca general cable o equivalente bajo tubo corrugado 25 mm de diámetro cero halógenos marca aiscan o equivalente, con parte proporcional de cajas de empotrar de paso y derivación, fijaciones, accesorios de unión y derivación, bornas, totalmente conexionado e instalado.</t>
   </si>
   <si>
-    <t xml:space="preserve">Extractores (11) y campana</t>
+    <t xml:space="preserve">Extractores (10) y campana</t>
   </si>
   <si>
     <t xml:space="preserve">16.05.25</t>
@@ -3790,7 +3790,7 @@
     <t xml:space="preserve">Opción 3 de cubiertas · IFC final (21-oct)</t>
   </si>
   <si>
-    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261022-0127.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (310,64 m²: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos, sin contar dos veces lo que se solapaba; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta, por detrás de la arista del faldón y no al borde del muro (Enrique 22-oct; 24,08 m en total). La unidad exterior de la aerotermia va en el hueco del muro grueso de la cubierta, junto al V12, ventilada y registrable desde la terraza (Enrique 22-oct); la puerta perforada contigua al V12 está en propuesta (hoja LO-G3b) y todavía no tiene partida. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement). IFC 22:38 (Enrique 21-oct, «el mortero es continuo»): los paños de revoco del mismo plano forman uno solo (con los cantos de losas y faldones) y la junta de poliestireno de las medianeras solo va contra la casa vecina: donde la medianera asoma por encima del vecino y lleva revoco, no hay junta. IFC 00:51 (22-oct): la barandilla del patio en cubierta pasa por detrás de la arista del faldón (−0,31 m) y la unidad exterior de la aerotermia, al muro grueso junto al V12. IFC 01:27 (22-oct): lleva además las instalaciones (tuberías, conductos, tubos eléctricos y suelo radiante como IfcFlowSegment con su diámetro orientativo y longitud; tomas, mecanismos, puntos de luz y de agua, desagües, bocas, llaves y equipos como IfcFlowTerminal, IfcFlowController…, agrupados por red en IfcSystem), sin medición en este presupuesto. Ventilación (Enrique 21/22-oct): cada boca de extracción lleva rejilla circular vista Ø125 de aluminio anodizado (tipo Mayfe) y extractor silencioso en línea de motor independiente (tipo Soler &amp; Palau) en el falso techo; 11 bocas en los planos LO-H5 y LO-H6, contadas en el modelo 3D (16.04.01, 16.04.02 y 16.05.24).</t>
+    <t xml:space="preserve">Enrique 21-oct: el proyecto se cierra con la opción 3 de cubiertas y el presupuesto se mide con el IFC final (lodosa_bim_20261022-0127.ifc, «basico op3»). Cambia respecto a la opción 2: no hay faldón ventilado de C. del Peso, ni celosía de tramex, ni almacenaje en cubierta (14.06 a 0); en la esquina SO, el faldón de C. del Peso sube desde el alero (+9,70) hasta la esquina del patio (+10,295) y desde la limatesa (de la esquina del alero en la medianera oeste a la esquina del patio) un faldón al 21,3 % vierte a la medianera oeste hasta el final del patio, con canalón junto a la medianera (5,67 m en 07.06); la cubierta plana queda en 29,31 m². Cada alero es parte de su faldón (un solo elemento IfcRoof en el IFC), pero vuela 200 mm sin aislamiento (regla de Enrique del 21-oct): losa de Ytong y XPS se miden sin los aleros (82,06 m²); OSB, lámina, rastreles y teja, con ellos (88,37 m²). El lucernario de la escalera es el V12 (2,87 m, alféizar a +9,84 y cabeza en el plano del faldón, de 1,80 a 0,94 m de alto, 3,93 m²); para cumplir el control solar sin estor lleva vidrio de control solar (g ≤ 0,35): sin estor, qsol;jul ≈ 2,30 &gt; 2,00; con el vidrio de control solar, ≈ 1,88. El revoco se mide como piel continua de arriba abajo (310,64 m²: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos, sin contar dos veces lo que se solapaba; huecos descontados, con mochetas y dinteles). La barandilla del borde norte del patio va recta, por detrás de la arista del faldón y no al borde del muro (Enrique 22-oct; 24,08 m en total). La unidad exterior de la aerotermia va en el hueco del muro grueso de la cubierta, junto al V12, ventilada y registrable desde la terraza (Enrique 22-oct); la puerta perforada contigua al V12 está en propuesta (hoja LO-G3b) y todavía no tiene partida. DB-HE recalculado (Anejo 04_2): K ≈ 0,51 &lt; 0,53. Comprobación del IFC: esquema IFC2X3 válido, sin GUID repetidos, 4 plantas, 17 recintos, mediciones en la descripción de cada elemento. Enrique 21-oct 18:50: la geometría de cubiertas sale de su planta de cubiertas (la limatesa va de la esquina del patio a la esquina del alero en la medianera oeste, faldón al 21 %; el borde norte del faldón llega 22 cm más allá). El muro de 45 cm del baño de segunda y de la cocina es de carga de 20 cm con trasdosado de 7 cm (baldosa hacia el baño). Corregido en este IFC respecto al de las 16:58: la junta de las medianeras y la baldosa de los tabiques de baño salen como capas, cada alero va dentro de su faldón, y los 38 muros de segunda cuya fábrica se para bajo el zuncho de coronación se exportan partidos (el muro entero hasta 250 mm por debajo de la coronación más baja y, encima, las capas junto al zuncho y la cuña inclinada, como muros aparte «· coronación» sin medición propia) para que todos los muros lleven su juego de capas; los volúmenes por material no cambian. Quedan, sin efecto en el presupuesto: (1) el nombre del V12 lleva un carácter de control en lugar del guion; (2) las carpinterías no abren hueco en los muros (sin IfcOpeningElement). IFC 22:38 (Enrique 21-oct, «el mortero es continuo»): los paños de revoco del mismo plano forman uno solo (con los cantos de losas y faldones) y la junta de poliestireno de las medianeras solo va contra la casa vecina: donde la medianera asoma por encima del vecino y lleva revoco, no hay junta. IFC 00:51 (22-oct): la barandilla del patio en cubierta pasa por detrás de la arista del faldón (−0,31 m) y la unidad exterior de la aerotermia, al muro grueso junto al V12. IFC 01:27 (22-oct): lleva además las instalaciones (tuberías, conductos, tubos eléctricos y suelo radiante como IfcFlowSegment con su diámetro orientativo y longitud; tomas, mecanismos, puntos de luz y de agua, desagües, bocas, llaves y equipos como IfcFlowTerminal, IfcFlowController…, agrupados por red en IfcSystem), sin medición en este presupuesto. Ventilación (Enrique 21/22-oct): cada boca de extracción lleva rejilla circular vista Ø125 de aluminio anodizado (tipo Mayfe) y extractor silencioso en línea de motor independiente (tipo Soler &amp; Palau) en el falso techo; 10 bocas en los planos LO-H5 y LO-H6, contadas en el modelo 3D (16.04.01, 16.04.02 y 16.05.24); la salida de aire de la cámara Cupolex de planta baja no es boca (va por su conducto a cubierta, 04.06–04.07).</t>
   </si>
   <si>
     <t xml:space="preserve">MEDICIONES DEL MODELO BIM FRENTE A LA PROPUESTA DE OCTUBRE</t>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C7/$C$50)</f>
-        <v>0.00247282685747316</v>
+        <v>0.00247483345957182</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C8/$C$50)</f>
-        <v>0.0241071563147481</v>
+        <v>0.0241267183274737</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C9/$C$50)</f>
-        <v>0.0250175260176693</v>
+        <v>0.0250378267597365</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C10/$C$50)</f>
-        <v>0.00376164387676886</v>
+        <v>0.0037646963033772</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C14/$C$50)</f>
-        <v>0.003971517662721</v>
+        <v>0.00397474039368286</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C16/$C$50)</f>
-        <v>0.0130384543514268</v>
+        <v>0.0130490345462293</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C17/$C$50)</f>
-        <v>0.0168156895935056</v>
+        <v>0.0168293348666985</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C18/$C$50)</f>
-        <v>0.186481056607889</v>
+        <v>0.186632378678183</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C21/$C$50)</f>
-        <v>0.145358506323336</v>
+        <v>0.145476459055436</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C22/$C$50)</f>
-        <v>0.0373228489486997</v>
+        <v>0.0373531349781491</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C23/$C$50)</f>
-        <v>0.019538600912855</v>
+        <v>0.0195544557218879</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C24/$C$50)</f>
-        <v>0.00953493707171901</v>
+        <v>0.00954267429953217</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C25/$C$50)</f>
-        <v>0.0564627934377318</v>
+        <v>0.0565086107821473</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C26/$C$50)</f>
-        <v>0.0741338030217</v>
+        <v>0.0741939596979654</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C27/$C$50)</f>
-        <v>0.0274229545938194</v>
+        <v>0.027445207246921</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C28/$C$50)</f>
-        <v>0.136376479016759</v>
+        <v>0.136487143185654</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C29/$C$50)</f>
-        <v>0.0532065069590282</v>
+        <v>0.0532496819545618</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C30/$C$50)</f>
-        <v>0.0232478411990647</v>
+        <v>0.0232667059112457</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5022,11 +5022,11 @@
       </c>
       <c r="C31" s="8" t="n">
         <f aca="false">Presupuesto!K1073</f>
-        <v>46262.05</v>
+        <v>45949.51</v>
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C31/$C$50)</f>
-        <v>0.120014729040879</v>
+        <v>0.119300655475168</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="C35" s="12" t="n">
         <f aca="false">SUMIFS(Presupuesto!$K$5:$K$1399,Presupuesto!$M$5:$M$1399,"P",Presupuesto!$O$5:$O$1399,"16.04")</f>
-        <v>4334.5</v>
+        <v>4031.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="C36" s="12" t="n">
         <f aca="false">SUMIFS(Presupuesto!$K$5:$K$1399,Presupuesto!$M$5:$M$1399,"P",Presupuesto!$O$5:$O$1399,"16.05")</f>
-        <v>12535.07</v>
+        <v>12525.53</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C38/$C$50)</f>
-        <v>0.00395491454492009</v>
+        <v>0.00395812380310244</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C41/$C$50)</f>
-        <v>0.00713425594956512</v>
+        <v>0.00714004511871684</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="D42" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C42/$C$50)</f>
-        <v>0.0106249576977204</v>
+        <v>0.0106335794345598</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="C48" s="10" t="n">
         <f aca="false">C14+C15+C16+C17+C18+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C38+C41+C42</f>
-        <v>364130.49</v>
+        <v>363817.95</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="C50" s="14" t="n">
         <f aca="false">C11+C48</f>
-        <v>385469.77</v>
+        <v>385157.23</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="C52" s="15" t="n">
         <f aca="false">ROUND(C50*D52,2)</f>
-        <v>19273.49</v>
+        <v>19257.86</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>0.05</v>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="C53" s="15" t="n">
         <f aca="false">ROUND(C50*D53,2)</f>
-        <v>19273.49</v>
+        <v>19257.86</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>0.05</v>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">C50+C52+C53</f>
-        <v>424016.75</v>
+        <v>423672.95</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="C56" s="15" t="n">
         <f aca="false">ROUND(C48*(1+$D$52+$D$53)*D56,2)</f>
-        <v>40054.35</v>
+        <v>40019.97</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>0.1</v>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C57" s="14" t="n">
         <f aca="false">C54+C55+C56</f>
-        <v>469000.47</v>
+        <v>468622.29</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="C61" s="15" t="n">
         <f aca="false">C50/C60</f>
-        <v>1097.64157981662</v>
+        <v>1096.75160886155</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18807,11 +18807,11 @@
         <v>800</v>
       </c>
       <c r="D856" s="28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H856" s="29" t="n">
         <f aca="false">IF(COUNT(D856:G856)=0,0,D856*IF(E856="",1,E856)*IF(F856="",1,F856)*IF(G856="",1,G856))</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M856" s="23"/>
       <c r="N856" s="23"/>
@@ -18821,14 +18821,14 @@
       <c r="H857" s="30"/>
       <c r="I857" s="31" t="n">
         <f aca="false">ROUND(SUM(H856:H856),2)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J857" s="32" t="n">
         <v>38</v>
       </c>
       <c r="K857" s="31" t="n">
         <f aca="false">ROUND(I857*J857,2)</f>
-        <v>418</v>
+        <v>380</v>
       </c>
       <c r="L857" s="33" t="s">
         <v>801</v>
@@ -18870,11 +18870,11 @@
         <v>805</v>
       </c>
       <c r="D860" s="28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H860" s="29" t="n">
         <f aca="false">IF(COUNT(D860:G860)=0,0,D860*IF(E860="",1,E860)*IF(F860="",1,F860)*IF(G860="",1,G860))</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M860" s="23"/>
       <c r="N860" s="23"/>
@@ -18884,14 +18884,14 @@
       <c r="H861" s="30"/>
       <c r="I861" s="31" t="n">
         <f aca="false">ROUND(SUM(H860:H860),2)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J861" s="32" t="n">
         <v>265</v>
       </c>
       <c r="K861" s="31" t="n">
         <f aca="false">ROUND(I861*J861,2)</f>
-        <v>2915</v>
+        <v>2650</v>
       </c>
       <c r="L861" s="33" t="s">
         <v>806</v>
@@ -20670,11 +20670,11 @@
         <v>904</v>
       </c>
       <c r="D974" s="28" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H974" s="29" t="n">
         <f aca="false">IF(COUNT(D974:G974)=0,0,D974*IF(E974="",1,E974)*IF(F974="",1,F974)*IF(G974="",1,G974))</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M974" s="23"/>
       <c r="N974" s="23"/>
@@ -20684,14 +20684,14 @@
       <c r="H975" s="30"/>
       <c r="I975" s="31" t="n">
         <f aca="false">ROUND(SUM(H974:H974),2)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J975" s="32" t="n">
         <v>9.54</v>
       </c>
       <c r="K975" s="31" t="n">
         <f aca="false">ROUND(I975*J975,2)</f>
-        <v>114.48</v>
+        <v>104.94</v>
       </c>
       <c r="L975" s="33" t="s">
         <v>212</v>
@@ -22241,7 +22241,7 @@
       </c>
       <c r="K1073" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$1072,$M$5:$M$1072,"P",$N$5:$N$1072,"16")</f>
-        <v>46262.05</v>
+        <v>45949.51</v>
       </c>
       <c r="M1073" s="23"/>
       <c r="N1073" s="23"/>
@@ -30042,7 +30042,7 @@
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">Resumen!C48</f>
-        <v>364130.49</v>
+        <v>363817.95</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="J64" s="45" t="n">
         <f aca="false">J63-J62</f>
-        <v>4927.46999999997</v>
+        <v>4614.92999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Visor: lodosa (2026-10-24 00:10)
</commit_message>
<xml_diff>
--- a/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
+++ b/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
@@ -913,7 +913,7 @@
     <t xml:space="preserve">Hormigón de limpieza HM-20/P/20/I de 10 cm de espesor en el fondo de zapatas y vigas de atado, vertido y nivelado.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bajo zapatas corridas (ZC-1 38,9 × 0,80; ZC-2 15,4 × 0,70), aisladas (5,78 m²) y vigas de atado (26,0 × 0,40): plano LO-E1</t>
+    <t xml:space="preserve">Medición del IFC con la estructura del ingeniero (lodosa_bim_20261024-0000.ifc): planta de zapatas corridas 43,43 + aisladas 4,71 + vigas de atado 8,37 m²</t>
   </si>
   <si>
     <t xml:space="preserve">05.01.02</t>
@@ -925,7 +925,7 @@
     <t xml:space="preserve">Zapatas corridas bajo los muros (ZC-1 80×50 excéntricas en las medianeras, ZC-2 70×40), zapatas aisladas bajo los pilares (Z-P6 130×130×50, Z-P7 110×110×50, Z-P8 y Z-P9 120×120×50) y vigas de atado y centradoras 40×40 (VA-1 40×50 bajo el portón), de hormigón armado HA-25/B/20/XC2 con acero B 500 S según el cuadro de cimentación del plano LO-E1, incluso encofrado donde sea necesario, vertido, vibrado y curado.</t>
   </si>
   <si>
-    <t xml:space="preserve">Plano LO-E1: zapatas corridas 19,87 m³ (ZC-1 38,9 m × 0,80 × 0,50; ZC-2 15,4 m × 0,70 × 0,40, longitudes estimadas sobre la planta) + aisladas 2,89 m³ + vigas de atado 4,38 m³ (40×40 en 20,6 m; VA-1 40×50 en 5,4 m)</t>
+    <t xml:space="preserve">Medición del IFC (lodosa_bim_20261024-0000.ifc): zapatas corridas 20,71 m³ (ZC-1 80×50 excéntricas en medianeras, ZC-2 70×40, trazadas bajo los muros con zócalo) + aisladas 2,35 m³ + vigas de atado 3,51 m³</t>
   </si>
   <si>
     <t xml:space="preserve">Mismo precio que la zapata corrida de la propuesta; contrastar con el aparejador</t>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C7/$C$50)</f>
-        <v>0.00241608343041264</v>
+        <v>0.00241682546628162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C8/$C$50)</f>
-        <v>0.0235539745738396</v>
+        <v>0.0235612085516778</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C9/$C$50)</f>
-        <v>0.0244434542186155</v>
+        <v>0.0244509613765074</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4739,7 +4739,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C10/$C$50)</f>
-        <v>0.00367532624223492</v>
+        <v>0.00367645502109563</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C14/$C$50)</f>
-        <v>0.0038803840994741</v>
+        <v>0.00388157585641055</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C16/$C$50)</f>
-        <v>0.0127392637383695</v>
+        <v>0.0127431762649484</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C17/$C$50)</f>
-        <v>0.0164298235742015</v>
+        <v>0.0164348695582349</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4834,11 +4834,11 @@
       </c>
       <c r="C18" s="8" t="n">
         <f aca="false">Presupuesto!K286</f>
-        <v>81248.38</v>
+        <v>81127.25</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C18/$C$50)</f>
-        <v>0.205940898726259</v>
+        <v>0.205697024558745</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">SUMIFS(Presupuesto!$K$5:$K$1399,Presupuesto!$M$5:$M$1399,"P",Presupuesto!$O$5:$O$1399,"05.01")</f>
-        <v>18669.18</v>
+        <v>18548.05</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C21/$C$50)</f>
-        <v>0.142022995882621</v>
+        <v>0.142066614474528</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C22/$C$50)</f>
-        <v>0.0364664095459122</v>
+        <v>0.0364776092352753</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C23/$C$50)</f>
-        <v>0.019090252832029</v>
+        <v>0.0190961158962638</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C24/$C$50)</f>
-        <v>0.00931614091758449</v>
+        <v>0.00931900212288655</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C25/$C$50)</f>
-        <v>0.0551671538374968</v>
+        <v>0.0551840969638896</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C26/$C$50)</f>
-        <v>0.07243267055795</v>
+        <v>0.072454916329335</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C27/$C$50)</f>
-        <v>0.0267936859415983</v>
+        <v>0.0268019149107558</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C28/$C$50)</f>
-        <v>0.13324707722849</v>
+        <v>0.133288000530018</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C29/$C$50)</f>
-        <v>0.051985588665598</v>
+        <v>0.0520015546587315</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C30/$C$50)</f>
-        <v>0.0227143779776479</v>
+        <v>0.0227213540956863</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C31/$C$50)</f>
-        <v>0.116468579255749</v>
+        <v>0.116504349487161</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C38/$C$50)</f>
-        <v>0.0038641619698532</v>
+        <v>0.0038653487445933</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C41/$C$50)</f>
-        <v>0.00697054770979016</v>
+        <v>0.00697268852842332</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5182,7 +5182,7 @@
       </c>
       <c r="D42" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C42/$C$50)</f>
-        <v>0.010381149074274</v>
+        <v>0.0103843373685512</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="C48" s="10" t="n">
         <f aca="false">C14+C15+C16+C17+C18+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C38+C41+C42</f>
-        <v>373183.52</v>
+        <v>373062.39</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="C50" s="14" t="n">
         <f aca="false">C11+C48</f>
-        <v>394522.8</v>
+        <v>394401.67</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="C52" s="15" t="n">
         <f aca="false">ROUND(C50*D52,2)</f>
-        <v>19726.14</v>
+        <v>19720.08</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>0.05</v>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="C53" s="15" t="n">
         <f aca="false">ROUND(C50*D53,2)</f>
-        <v>19726.14</v>
+        <v>19720.08</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>0.05</v>
@@ -5293,7 +5293,7 @@
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">C50+C52+C53</f>
-        <v>433975.08</v>
+        <v>433841.83</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C56" s="15" t="n">
         <f aca="false">ROUND(C48*(1+$D$52+$D$53)*D56,2)</f>
-        <v>41050.19</v>
+        <v>41036.86</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>0.1</v>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="C57" s="14" t="n">
         <f aca="false">C54+C55+C56</f>
-        <v>479954.64</v>
+        <v>479808.06</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="C61" s="15" t="n">
         <f aca="false">C50/C60</f>
-        <v>1123.420468136</v>
+        <v>1123.0755453044</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8764,7 +8764,7 @@
         <v>1</v>
       </c>
       <c r="E218" s="28" t="n">
-        <v>58.08</v>
+        <v>56.51</v>
       </c>
       <c r="F218" s="28"/>
       <c r="G218" s="28" t="n">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="H218" s="29" t="n">
         <f aca="false">IF(COUNT(D218:G218)=0,0,D218*IF(E218="",1,E218)*IF(F218="",1,F218)*IF(G218="",1,G218))</f>
-        <v>5.808</v>
+        <v>5.651</v>
       </c>
       <c r="M218" s="23"/>
       <c r="N218" s="23"/>
@@ -8782,14 +8782,14 @@
       <c r="H219" s="30"/>
       <c r="I219" s="31" t="n">
         <f aca="false">ROUND(SUM(H218:H218),2)</f>
-        <v>5.81</v>
+        <v>5.65</v>
       </c>
       <c r="J219" s="32" t="n">
         <v>98</v>
       </c>
       <c r="K219" s="31" t="n">
         <f aca="false">ROUND(I219*J219,2)</f>
-        <v>569.38</v>
+        <v>553.7</v>
       </c>
       <c r="L219" s="33" t="s">
         <v>238</v>
@@ -8834,13 +8834,13 @@
         <v>1</v>
       </c>
       <c r="E222" s="28" t="n">
-        <v>27.14</v>
+        <v>26.57</v>
       </c>
       <c r="F222" s="28"/>
       <c r="G222" s="28"/>
       <c r="H222" s="29" t="n">
         <f aca="false">IF(COUNT(D222:G222)=0,0,D222*IF(E222="",1,E222)*IF(F222="",1,F222)*IF(G222="",1,G222))</f>
-        <v>27.14</v>
+        <v>26.57</v>
       </c>
       <c r="M222" s="23"/>
       <c r="N222" s="23"/>
@@ -8850,14 +8850,14 @@
       <c r="H223" s="30"/>
       <c r="I223" s="31" t="n">
         <f aca="false">ROUND(SUM(H222:H222),2)</f>
-        <v>27.14</v>
+        <v>26.57</v>
       </c>
       <c r="J223" s="32" t="n">
         <v>185</v>
       </c>
       <c r="K223" s="31" t="n">
         <f aca="false">ROUND(I223*J223,2)</f>
-        <v>5020.9</v>
+        <v>4915.45</v>
       </c>
       <c r="L223" s="33" t="s">
         <v>300</v>
@@ -9900,7 +9900,7 @@
       </c>
       <c r="K286" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$285,$M$5:$M$285,"P",$N$5:$N$285,"05")</f>
-        <v>81248.38</v>
+        <v>81127.25</v>
       </c>
       <c r="M286" s="23"/>
       <c r="N286" s="23"/>
@@ -30042,7 +30042,7 @@
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">Resumen!C48</f>
-        <v>373183.52</v>
+        <v>373062.39</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="J64" s="45" t="n">
         <f aca="false">J63-J62</f>
-        <v>13980.5</v>
+        <v>13859.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Visor: lodosa (2026-10-24 11:53)
</commit_message>
<xml_diff>
--- a/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
+++ b/datos/lodosa/presupuestos/Presupuesto_Conjunto_Lodosa_2026-10.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">DERRIBO Y VIVIENDA DE NUEVA PLANTA · C. ANCHA 34, LODOSA</t>
   </si>
   <si>
-    <t xml:space="preserve">Presupuesto conjunto (derribo + obra nueva) · propuesta de octubre de 2026, con las mediciones del modelo BIM del 14-oct y la opción 3 de cubiertas del IFC final (21-oct); con la estructura del ingeniero (23-oct)</t>
+    <t xml:space="preserve">Presupuesto conjunto (derribo + obra nueva) · propuesta de octubre de 2026, con las mediciones del modelo BIM del 14-oct y la opción 3 de cubiertas del IFC final (21-oct); con la estructura del ingeniero (23-oct) y el IFC del 24-oct (muros bajo rasante y revoco)</t>
   </si>
   <si>
     <t xml:space="preserve">Capítulo</t>
@@ -3838,7 +3838,7 @@
     <t xml:space="preserve">Cómo se mide en el BIM</t>
   </si>
   <si>
-    <t xml:space="preserve">Zócalo de 0,90 m bajo los muros de planta baja con el grueso que indica Enrique: 0,32 m en fachada a calle (7.9 m) y 0,21 m de media en el resto (58.5 m). Con el grueso de hormigón de cada muro del BIM sale 12.79 m³</t>
+    <t xml:space="preserve">Zócalo de 0,90 m bajo los muros de planta baja con el grueso que indica Enrique: 0,32 m en fachada a calle (7.9 m) y 0,21 m de media en el resto (58.5 m). Con el grueso de hormigón de cada muro del BIM sale 12.79 m³ · BIM 24-oct: + muros de hormigón bajo rasante (MC) de la cara superior de la cimentación al suelo de planta baja, 23 tramos, 74,05 m de eje: 14.37 m³ (al precio del zócalo)</t>
   </si>
   <si>
     <t xml:space="preserve">Superficie de estancias y escalera de planta baja (garaje incluido)</t>
@@ -3928,7 +3928,7 @@
     <t xml:space="preserve">Patio y porche 29.6 + terraza 11.1 + cubierta plana 49.3 m² · Partida nueva · Opción 2 de cubiertas (16-oct): patio y porche 29,6 + terraza 11,1 + cubierta plana descubierta 29,32 m² · Faldón de C. del Peso ventilado (Enrique 16-oct): +17,15 m² bajo el faldón · Opción 3 de cubiertas, IFC final (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 30,02 m² · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): patio y porche 29,65 + terraza 11,05 + cubierta plana 29,31 m²</t>
   </si>
   <si>
-    <t xml:space="preserve">Caras revocadas de muros exteriores y frentes de forjado · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro y +0,68 m² de frente de forjado · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): revoco continuo del IFC (piel vista de la casa, 34 paños de arriba abajo, regla de Enrique del 19 y 21-oct): caras 289,80 m² con los huecos descontados + mochetas y dinteles 18,68 m²; sin medianeras, bajo aleros ni zócalo. Sustituye a la medición por caras de muro (261,81) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): revoco continuo del IFC 20:01: paños de fachada 308,86 m² + cantos de losas y faldones que quedaban vistos 13,43 m² (patinillo, bordes de la cubierta plana, terraza de segunda, faldones sobre la terraza; Enrique 21-oct: el mortero es continuo) · IFC 22:38 (21-oct, mortero continuo): revoco continuo del IFC 22:38: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos (cara 291,79 m² + mochetas y dinteles 18,85 m²); −11,65 m² respecto al IFC 20:01, que contaba dos veces los cantos tapados por el paño</t>
+    <t xml:space="preserve">Caras revocadas de muros exteriores y frentes de forjado · Opción 2 de cubiertas (16-oct): −1,50 m² de muro de quiebro y +0,68 m² de frente de forjado · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): revoco continuo del IFC (piel vista de la casa, 34 paños de arriba abajo, regla de Enrique del 19 y 21-oct): caras 289,80 m² con los huecos descontados + mochetas y dinteles 18,68 m²; sin medianeras, bajo aleros ni zócalo. Sustituye a la medición por caras de muro (261,81) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): revoco continuo del IFC 20:01: paños de fachada 308,86 m² + cantos de losas y faldones que quedaban vistos 13,43 m² (patinillo, bordes de la cubierta plana, terraza de segunda, faldones sobre la terraza; Enrique 21-oct: el mortero es continuo) · IFC 22:38 (21-oct, mortero continuo): revoco continuo del IFC 22:38: cada plano de fachada es un solo paño, con los cantos de losas y faldones que quedaban vistos (cara 291,79 m² + mochetas y dinteles 18,85 m²); −11,65 m² respecto al IFC 20:01, que contaba dos veces los cantos tapados por el paño · IFC 24-oct 11:33–11:50 (captura «mortero»): revoco de la cámara bajo el faldón C. del Peso (5,39 m²), esquinas cerradas y pared del patio en un solo paño: 316.10 m²</t>
   </si>
   <si>
     <t xml:space="preserve">Paredes 726.4 m² (incluye 27.6 m² de baños y aseos por encima de 2,28 m) y techos sin falso techo 214.4 m² · Opción 2 de cubiertas (16-oct): paredes: +8,09 medianera M2, +5,08 muro M13 (dos caras), −4,72 tabique T2 (dos caras), −1,50 quiebro; techos: −8,52 m² que pasan a falso techo · Opción 3 de cubiertas, IFC final (21-oct): paredes −0,80 m² (cambios de muros de segunda) y techos +8,89 m²: bajo el faldón de la escalera ya no hay falso techo (+8,52) y el faldón a la medianera oeste tiene más superficie en pendiente que la cubierta plana a la que sustituye (+0,37) · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): +2,84 m² de yeso en paredes (muros de segunda remedidos y trasdosado M13t)</t>
@@ -3982,7 +3982,7 @@
     <t xml:space="preserve">Yeso de paredes y techos más falsos techos · Opción 2 de cubiertas (16-oct): yeso 939,20 + falsos techos 96,96 · Opción 3 de cubiertas, IFC final (21-oct): yeso 947,29 + falsos techos 88,43 · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): yeso 950,13 + falsos techos 88,49</t>
   </si>
   <si>
-    <t xml:space="preserve">Igual que el revoco · Opción 2 de cubiertas (16-oct): igual que el revoco · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): igual que el revoco · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): igual que el revoco · IFC 22:38 (21-oct, mortero continuo): igual que el revoco</t>
+    <t xml:space="preserve">Igual que el revoco · Opción 2 de cubiertas (16-oct): igual que el revoco · +13,89 m² de los piñones del faldón de C. del Peso · Celosía de tramex en el frente del faldón ventilado (Enrique 16-oct): −6,42 m² del piñón norte · Opción 3 de cubiertas, IFC final (21-oct): igual que el revoco · Opción 3, planta de cubiertas de Enrique e IFC 20:01 (21-oct): igual que el revoco · IFC 22:38 (21-oct, mortero continuo): igual que el revoco · IFC 24-oct 11:33–11:50 (captura «mortero»): revoco de la cámara bajo el faldón C. del Peso (5,39 m²), esquinas cerradas y pared del patio en un solo paño: 316.10 m²</t>
   </si>
   <si>
     <t xml:space="preserve">Total de las partidas medidas con el BIM</t>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C7/$C$50)</f>
-        <v>0.00241682546628162</v>
+        <v>0.00238382074948405</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C8/$C$50)</f>
-        <v>0.0235612085516778</v>
+        <v>0.0232394513430974</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C9/$C$50)</f>
-        <v>0.0244509613765074</v>
+        <v>0.0241170535015206</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4739,7 +4739,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C10/$C$50)</f>
-        <v>0.00367645502109563</v>
+        <v>0.00362624851736453</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C14/$C$50)</f>
-        <v>0.00388157585641055</v>
+        <v>0.00382856817602301</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C16/$C$50)</f>
-        <v>0.0127431762649484</v>
+        <v>0.0125691525592261</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C17/$C$50)</f>
-        <v>0.0164348695582349</v>
+        <v>0.0162104312514799</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4834,11 +4834,11 @@
       </c>
       <c r="C18" s="8" t="n">
         <f aca="false">Presupuesto!K286</f>
-        <v>81127.25</v>
+        <v>86385.23</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C18/$C$50)</f>
-        <v>0.205697024558745</v>
+        <v>0.216037456696341</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">SUMIFS(Presupuesto!$K$5:$K$1399,Presupuesto!$M$5:$M$1399,"P",Presupuesto!$O$5:$O$1399,"05.01")</f>
-        <v>18548.05</v>
+        <v>23806.03</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C21/$C$50)</f>
-        <v>0.142066614474528</v>
+        <v>0.140126520561029</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C22/$C$50)</f>
-        <v>0.0364776092352753</v>
+        <v>0.0359794627290176</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C23/$C$50)</f>
-        <v>0.0190961158962638</v>
+        <v>0.0188353350058425</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C24/$C$50)</f>
-        <v>0.00931900212288655</v>
+        <v>0.00919173971598422</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C25/$C$50)</f>
-        <v>0.0551840969638896</v>
+        <v>0.0544304904178509</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4954,11 +4954,11 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">Presupuesto!K545</f>
-        <v>28576.34</v>
+        <v>28737.74</v>
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C26/$C$50)</f>
-        <v>0.072454916329335</v>
+        <v>0.0718690945292464</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C27/$C$50)</f>
-        <v>0.0268019149107558</v>
+        <v>0.0264359018810176</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C28/$C$50)</f>
-        <v>0.133288000530018</v>
+        <v>0.131467789359877</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C29/$C$50)</f>
-        <v>0.0520015546587315</v>
+        <v>0.0512914096323364</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5018,11 +5018,11 @@
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">Presupuesto!K676</f>
-        <v>8961.34</v>
+        <v>9002.57</v>
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C30/$C$50)</f>
-        <v>0.0227213540956863</v>
+        <v>0.0225141766310141</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C31/$C$50)</f>
-        <v>0.116504349487161</v>
+        <v>0.114913339662846</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C38/$C$50)</f>
-        <v>0.0038653487445933</v>
+        <v>0.00381256266532567</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C41/$C$50)</f>
-        <v>0.00697268852842332</v>
+        <v>0.00687746791220217</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5182,7 +5182,7 @@
       </c>
       <c r="D42" s="9" t="n">
         <f aca="false">IF($C$50=0,0,C42/$C$50)</f>
-        <v>0.0103843373685512</v>
+        <v>0.0102425265018746</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="C48" s="10" t="n">
         <f aca="false">C14+C15+C16+C17+C18+C21+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C38+C41+C42</f>
-        <v>373062.39</v>
+        <v>378523</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="C50" s="14" t="n">
         <f aca="false">C11+C48</f>
-        <v>394401.67</v>
+        <v>399862.28</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="C52" s="15" t="n">
         <f aca="false">ROUND(C50*D52,2)</f>
-        <v>19720.08</v>
+        <v>19993.11</v>
       </c>
       <c r="D52" s="16" t="n">
         <v>0.05</v>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="C53" s="15" t="n">
         <f aca="false">ROUND(C50*D53,2)</f>
-        <v>19720.08</v>
+        <v>19993.11</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>0.05</v>
@@ -5293,7 +5293,7 @@
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">C50+C52+C53</f>
-        <v>433841.83</v>
+        <v>439848.5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C56" s="15" t="n">
         <f aca="false">ROUND(C48*(1+$D$52+$D$53)*D56,2)</f>
-        <v>41036.86</v>
+        <v>41637.53</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>0.1</v>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="C57" s="14" t="n">
         <f aca="false">C54+C55+C56</f>
-        <v>479808.06</v>
+        <v>486415.4</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="C61" s="15" t="n">
         <f aca="false">C50/C60</f>
-        <v>1123.0755453044</v>
+        <v>1138.62486474173</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8903,13 +8903,13 @@
       </c>
       <c r="E226" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E6</f>
-        <v>13.34</v>
+        <v>27.71</v>
       </c>
       <c r="F226" s="28"/>
       <c r="G226" s="28"/>
       <c r="H226" s="29" t="n">
         <f aca="false">IF(COUNT(D226:G226)=0,0,D226*IF(E226="",1,E226)*IF(F226="",1,F226)*IF(G226="",1,G226))</f>
-        <v>13.34</v>
+        <v>27.71</v>
       </c>
       <c r="M226" s="23"/>
       <c r="N226" s="23"/>
@@ -8919,14 +8919,14 @@
       <c r="H227" s="30"/>
       <c r="I227" s="31" t="n">
         <f aca="false">ROUND(SUM(H226:H226),2)</f>
-        <v>13.34</v>
+        <v>27.71</v>
       </c>
       <c r="J227" s="32" t="n">
         <v>365.9</v>
       </c>
       <c r="K227" s="31" t="n">
         <f aca="false">ROUND(I227*J227,2)</f>
-        <v>4881.11</v>
+        <v>10139.09</v>
       </c>
       <c r="L227" s="33" t="s">
         <v>212</v>
@@ -9900,7 +9900,7 @@
       </c>
       <c r="K286" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$285,$M$5:$M$285,"P",$N$5:$N$285,"05")</f>
-        <v>81127.25</v>
+        <v>86385.23</v>
       </c>
       <c r="M286" s="23"/>
       <c r="N286" s="23"/>
@@ -13521,11 +13521,11 @@
       </c>
       <c r="E519" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E38</f>
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="H519" s="29" t="n">
         <f aca="false">IF(COUNT(D519:G519)=0,0,D519*IF(E519="",1,E519)*IF(F519="",1,F519)*IF(G519="",1,G519))</f>
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="M519" s="23"/>
       <c r="N519" s="23"/>
@@ -13559,14 +13559,14 @@
       <c r="H522" s="30"/>
       <c r="I522" s="31" t="n">
         <f aca="false">ROUND(SUM(H519:H521),2)</f>
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="J522" s="32" t="n">
         <v>29.56</v>
       </c>
       <c r="K522" s="31" t="n">
         <f aca="false">ROUND(I522*J522,2)</f>
-        <v>9182.52</v>
+        <v>9343.92</v>
       </c>
       <c r="L522" s="33" t="s">
         <v>212</v>
@@ -13904,7 +13904,7 @@
       </c>
       <c r="K545" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$544,$M$5:$M$544,"P",$N$5:$N$544,"11")</f>
-        <v>28576.34</v>
+        <v>28737.74</v>
       </c>
       <c r="M545" s="23"/>
       <c r="N545" s="23"/>
@@ -15924,11 +15924,11 @@
       </c>
       <c r="E674" s="35" t="n">
         <f aca="false">'Mediciones BIM'!E58</f>
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="H674" s="29" t="n">
         <f aca="false">IF(COUNT(D674:G674)=0,0,D674*IF(E674="",1,E674)*IF(F674="",1,F674)*IF(G674="",1,G674))</f>
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="M674" s="23"/>
       <c r="N674" s="23"/>
@@ -15938,14 +15938,14 @@
       <c r="H675" s="30"/>
       <c r="I675" s="31" t="n">
         <f aca="false">ROUND(SUM(H674:H674),2)</f>
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="J675" s="32" t="n">
         <v>7.55</v>
       </c>
       <c r="K675" s="31" t="n">
         <f aca="false">ROUND(I675*J675,2)</f>
-        <v>2345.33</v>
+        <v>2386.56</v>
       </c>
       <c r="L675" s="33" t="s">
         <v>212</v>
@@ -15964,7 +15964,7 @@
       </c>
       <c r="K676" s="14" t="n">
         <f aca="false">SUMIFS($K$5:$K$675,$M$5:$M$675,"P",$N$5:$N$675,"15")</f>
-        <v>8961.34</v>
+        <v>9002.57</v>
       </c>
       <c r="M676" s="23"/>
       <c r="N676" s="23"/>
@@ -27538,15 +27538,15 @@
         <v>20.07</v>
       </c>
       <c r="E6" s="42" t="n">
-        <v>13.34</v>
+        <v>27.71</v>
       </c>
       <c r="F6" s="29" t="n">
         <f aca="false">E6-D6</f>
-        <v>-6.73</v>
+        <v>7.64</v>
       </c>
       <c r="G6" s="43" t="n">
         <f aca="false">IF(D6=0,"-",F6/D6)</f>
-        <v>-0.335326357747882</v>
+        <v>0.380667663178874</v>
       </c>
       <c r="H6" s="44" t="n">
         <f aca="false">Presupuesto!J227</f>
@@ -27558,11 +27558,11 @@
       </c>
       <c r="J6" s="44" t="n">
         <f aca="false">Presupuesto!K227</f>
-        <v>4881.11</v>
+        <v>10139.09</v>
       </c>
       <c r="K6" s="29" t="n">
         <f aca="false">J6-I6</f>
-        <v>-2462.5</v>
+        <v>2795.48</v>
       </c>
       <c r="L6" s="26" t="s">
         <v>1270</v>
@@ -29041,15 +29041,15 @@
         <v>196.3</v>
       </c>
       <c r="E38" s="42" t="n">
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="F38" s="29" t="n">
         <f aca="false">E38-D38</f>
-        <v>114.34</v>
+        <v>119.8</v>
       </c>
       <c r="G38" s="43" t="n">
         <f aca="false">IF(D38=0,"-",F38/D38)</f>
-        <v>0.582475802343352</v>
+        <v>0.610290371879776</v>
       </c>
       <c r="H38" s="44" t="n">
         <f aca="false">Presupuesto!J522</f>
@@ -29061,11 +29061,11 @@
       </c>
       <c r="J38" s="44" t="n">
         <f aca="false">Presupuesto!K522</f>
-        <v>9182.52</v>
+        <v>9343.92</v>
       </c>
       <c r="K38" s="29" t="n">
         <f aca="false">J38-I38</f>
-        <v>3379.89</v>
+        <v>3541.29</v>
       </c>
       <c r="L38" s="26" t="s">
         <v>1300</v>
@@ -29981,15 +29981,15 @@
         <v>196.3</v>
       </c>
       <c r="E58" s="42" t="n">
-        <v>310.64</v>
+        <v>316.1</v>
       </c>
       <c r="F58" s="29" t="n">
         <f aca="false">E58-D58</f>
-        <v>114.34</v>
+        <v>119.8</v>
       </c>
       <c r="G58" s="43" t="n">
         <f aca="false">IF(D58=0,"-",F58/D58)</f>
-        <v>0.582475802343352</v>
+        <v>0.610290371879776</v>
       </c>
       <c r="H58" s="44" t="n">
         <f aca="false">Presupuesto!J675</f>
@@ -30001,11 +30001,11 @@
       </c>
       <c r="J58" s="44" t="n">
         <f aca="false">Presupuesto!K675</f>
-        <v>2345.33</v>
+        <v>2386.56</v>
       </c>
       <c r="K58" s="29" t="n">
         <f aca="false">J58-I58</f>
-        <v>863.26</v>
+        <v>904.49</v>
       </c>
       <c r="L58" s="26" t="s">
         <v>1318</v>
@@ -30021,11 +30021,11 @@
       </c>
       <c r="J60" s="45" t="n">
         <f aca="false">SUM(J6:J58)</f>
-        <v>225584.27</v>
+        <v>231044.88</v>
       </c>
       <c r="K60" s="45" t="n">
         <f aca="false">SUM(K6:K58)</f>
-        <v>25024.42</v>
+        <v>30485.03</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">Resumen!C48</f>
-        <v>373062.39</v>
+        <v>378523</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="J64" s="45" t="n">
         <f aca="false">J63-J62</f>
-        <v>13859.37</v>
+        <v>19319.9799999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>